<commit_message>
Update e-CVT ratio benchmark and UX materials
</commit_message>
<xml_diff>
--- a/research-mgu/03_analysis/网页重点内容提取_后续与AI对比.xlsx
+++ b/research-mgu/03_analysis/网页重点内容提取_后续与AI对比.xlsx
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="722" uniqueCount="628">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="774" uniqueCount="634">
   <si>
     <t>SourceID</t>
   </si>
@@ -310,6 +310,11 @@
     <t>E-MOUNTAINBIKE 对 Gobao X1P 的 Eurobike 2026 深度报道；补充 X1P E-CVT gearbox motor、150 Nm 级高输出、无后拨/飞轮思路、eMTB 场景和媒体试骑/评估语境</t>
   </si>
   <si>
+    <t>我们已经在全新Hepha Urban X上测试了另一个令人兴奋的功能。电机实现可控再生，停止踩踏后会轻柔减速。通过倒退，制动效果可以进一步增强。实际上，它已经出乎意料地表现良好，尤其是在较长的下坡上带来了明显的好处。不过，为了实现真正自然的骑行体验，系统在某些情况下仍需进一步打磨，比如过弯时。
+最引人注目的是即时且清晰的动力传输。即使在低踏频下，扭矩依然充足，加速极快且可控，最高可达25公里/小时的辅助限制。由于没有换挡，动力输出始终稳定且异常平稳。起始也非常简单且明确。
+更令人印象深刻的是噪音水平。虽然许多变速箱系统在负载下能清晰听到声音，但Gobao的传动依然出奇地安静。只有在约100转以上的节奏时，才会有轻微的电声嗡嗡声。尤其是直接与现有变速箱系统相比，X1P已经非常接近量产准备状态。</t>
+  </si>
+  <si>
     <t>Pinion - E-Drive MGU E1.9 / E1.12</t>
   </si>
   <si>
@@ -340,6 +345,12 @@
     <t>Auto.Shift、Auto.Shift.Pro、Pre.Select、Start.Select、传感器、目标踏频、手动覆盖、停车起步档、滑行预选档逻辑</t>
   </si>
   <si>
+    <t xml:space="preserve">Pinion E-Drive系统提供四个支持等级：“Eco”设计为最大续航，而“Fly”则允许骑手随时充分发挥系统强大的动力。然而，“流”和“灵活”两个等级是自适应骑行模式，设计得动态，能根据各种骑行情境和地形完美调整支撑量。精心调校的启动辅助装置帮助防止松散爬坡时的车轮打滑，车把上的增压按钮进一步完善了整体配置。此外，所有支持模式都可通过FIT电动自行车控制应用根据骑手个人偏好进行定制。
+除了提供调整和微调功率输出、启动、动力传输及所有Smart.Shift功能外，应用还提供简单明了的调校说明，指导用户完成调校过程。
+例如，结合FIT电动自行车控制应用，这些显示屏可以用来规划或显示通过Komoot的路线和方向。
+</t>
+  </si>
+  <si>
     <t>3.3-003</t>
   </si>
   <si>
@@ -355,6 +366,78 @@
     <t>Pinion MGU 在 eMTB 的场景叙事与 OEM 示例</t>
   </si>
   <si>
+    <r>
+      <t>Auto.Shift 是进一步简化电动自行车的先进方式。整个换挡过程都是自动化的，始终保持你偏好的步频。你设定一个想要的踏频，系统会根据地形或速度调整档位来保持这个踏频。Auto.Shift 对于长途旅行以及不断变化的城市交通状况来说都非常宝贵。
+自动换挡按钮在显示屏上以“A”表示，可随时开关，甚至在骑行中，只需长按E扳机即可。
+Auto.Shift.Pro，我们为您提供自动换挡与手动控制的完美结合。该模式专为动态骑行设计，允许你随时用TE1 E-Trigger覆盖自动换挡。一旦你手动介入并换挡，系统会记录随之而来的节奏变化，并相应调整换挡策略。Auto.Shift.Pro 非常适合注重自动换挡舒适性和手动自由的运动骑手。
+在多条路线上，你常常需要主动换挡并调整步频以应对即将到来的情况。自动变速箱对情况做出反应，但无法预见。Auto.Shift.Pro 就是解决办法。例如，接近陡坡时，你可能想在爬坡前提高踏频，以获得最佳动量。在 Auto.Shift.Pro 模式下，只需按TE1 E扳机上的按钮手动降一到两个档位。Auto.Shift.Pro 会自动接管较轻档的新踏频作为目标值，并根据爬坡时最佳调整换挡逻辑。如果新的踏频不再适合当前情况，你可以通过长按后部E-Trigger手柄迅速将其重置到预设值。 [</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="宋体"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>我认为Auto.Shift.Pro的问题是不能自动识别骑行者的意图。其实通过轮速、目标踏频、踩踏力矩和坡度可以理解此时骑行者的意图，系统自己做出判断</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="宋体"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>]
+Pre.Select是一种半自动换挡功能，用于在滑行时选择最佳档位以恢复踩踏。系统会持续监控你的速度，并自动调整档位，让你能平稳地开始踩踏。此功能特别适用于电动山地车的下坡骑行，确保你在下坡时始终处于正确的档位。 [</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="宋体"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>我认为这都是默认必要的，不应该单独设置为一个模式</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="宋体"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>]
+Start.Select是MGU内部半自动换挡的入门级变速器。你的电动自行车在停车时会自动换到预设的起步档位——例如在红绿灯处。这确保了开局轻松高效的过程。尤其是在频繁停停的情况下，Start.Select大大简化了重新起步，让你无需手动换挡就能专注于道路。 [</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="宋体"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>我认为这可以是通过大量的实验给一个默认的速比，来达到起步时踩下去的力矩值达到多大是一个舒适/时候的速比。可以做成每个品牌的初始默认值，也可以让客户自己试验选择一个起步的速比</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="宋体"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>]
+选用 Pinion 系统，换挡逻辑完全由你自定义：升档、降档，左右按键布局均可随心设置，TE1 电子变速指拨支持个性化调校。
+MGU配备了多种传感器，可监测踏板踩踏力度、曲柄位置、踏频、速度等。</t>
+    </r>
+  </si>
+  <si>
     <t>3.3-004</t>
   </si>
   <si>
@@ -487,6 +570,52 @@
     <t>外部电子/自动换挡生态；列出 3X3 Electric、Classified Powershift、enviolo AUTOMATiQ、Gearsensor GS、Rohloff E-14、Shimano Di2、TRP E.A.S.I. 等伙伴；含 M+、RollShift、Auto-downshift、适配车型与驱动单元边界</t>
   </si>
   <si>
+    <r>
+      <t>eShift 可适配 Classified 双速花鼓变速系统，</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="宋体"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>它会根据脚踏曲柄所处位置，在最优时机完成换挡操作</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="宋体"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">，城市电助力自行车是典型适配场景。
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="宋体"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>针对运动骑行模式，你可将目标踏频设置为 75 转 / 分钟及以上；若想要更休闲省力的骑行节奏，则可设定 60 转 / 分钟以下的踏频</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="宋体"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>。</t>
+    </r>
+  </si>
+  <si>
     <t>3.5-002</t>
   </si>
   <si>
@@ -499,6 +628,11 @@
     <t>E-MOUNTAINBIKE 对 Bosch eShift + TRP E.A.S.I. A12 的测试；用于评估外部自动换挡在 eMTB 场景中对 e-CVT MGU 的替代压力，以及与 Shimano/SRAM 自动换挡生态的竞争关系</t>
   </si>
   <si>
+    <t>按住博世Mini遥控器中键，可以将踏频设置在40到120转之间，每分钟5个增量。
+Roll-Shift 滑行换挡功能（无需踩踏即可完成变速）在三款变速系统上均可稳定运行，通过复杂越野路况时这项功能优势十分突出。
+但若在高难度林道开启自动变速进行运动骑行，博世、禧玛诺、速联三套系统都会很快达到性能上限，这类自动变速功能更适配平缓路况的长途休闲骑行。</t>
+  </si>
+  <si>
     <t>Shimano - AUTO SHIFT / FREE SHIFT / Di2 with EP platforms</t>
   </si>
   <si>
@@ -971,6 +1105,9 @@
   </si>
   <si>
     <t>横向解释 Avinox、Gobao、Owuru 等 eCVT 逻辑；用于机制框架、虚拟档/目标踏频、效率、低电/断电、法规和轻助力适配风险边界；不是单一产品规格源</t>
+  </si>
+  <si>
+    <t>我在Eurobike试驾Gabao eCVT时，把它调到最大助力模式（1500瓦），然后用后刹拉硬力冲刺。我强制它在手动模式下换挡（它有十二个“虚拟档位”），它毫无问题地换挡了。一旦你了解了电动CVT换挡的工作原理，这就不足为奇了——它只是调节传到电机的电信号。</t>
   </si>
   <si>
     <t>DJI / Avinox - Avinox MG Concept 扩展候选</t>
@@ -1961,7 +2098,7 @@
     <numFmt numFmtId="43" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="44" formatCode="_ &quot;￥&quot;* #,##0.00_ ;_ &quot;￥&quot;* \-#,##0.00_ ;_ &quot;￥&quot;* &quot;-&quot;??_ ;_ @_ "/>
   </numFmts>
-  <fonts count="25">
+  <fonts count="26">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -2139,6 +2276,14 @@
       <color theme="1"/>
       <name val="宋体"/>
       <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="宋体"/>
+      <charset val="134"/>
       <scheme val="minor"/>
     </font>
   </fonts>
@@ -2631,7 +2776,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -2687,6 +2832,9 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="6">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="6" applyFont="1">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -2748,6 +2896,53 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>19</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>27940</xdr:colOff>
+      <xdr:row>20</xdr:row>
+      <xdr:rowOff>85725</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="图片 1"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="14420850" y="33648650"/>
+          <a:ext cx="3723640" cy="2314575"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:ln w="9525">
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -3305,16 +3500,22 @@
       <c r="C13" s="17" t="s">
         <v>61</v>
       </c>
-      <c r="D13" s="17" t="s">
+      <c r="D13" s="21" t="s">
         <v>62</v>
       </c>
       <c r="E13" s="16" t="s">
         <v>63</v>
       </c>
-      <c r="F13" s="18"/>
+      <c r="F13" s="18" t="s">
+        <v>17</v>
+      </c>
       <c r="G13" s="18"/>
-      <c r="H13" s="15"/>
-      <c r="I13" s="15"/>
+      <c r="H13" s="15" t="s">
+        <v>17</v>
+      </c>
+      <c r="I13" s="15" t="s">
+        <v>17</v>
+      </c>
     </row>
     <row r="14" s="1" customFormat="1" ht="126" customHeight="1" spans="1:10">
       <c r="A14" s="16" t="s">
@@ -3326,16 +3527,22 @@
       <c r="C14" s="17" t="s">
         <v>13</v>
       </c>
-      <c r="D14" s="17" t="s">
+      <c r="D14" s="20" t="s">
         <v>14</v>
       </c>
       <c r="E14" s="16" t="s">
         <v>65</v>
       </c>
-      <c r="F14" s="18"/>
+      <c r="F14" s="18" t="s">
+        <v>17</v>
+      </c>
       <c r="G14" s="18"/>
-      <c r="H14" s="15"/>
-      <c r="I14" s="15"/>
+      <c r="H14" s="15" t="s">
+        <v>17</v>
+      </c>
+      <c r="I14" s="15" t="s">
+        <v>17</v>
+      </c>
     </row>
     <row r="15" s="1" customFormat="1" ht="283.5" customHeight="1" spans="1:10">
       <c r="A15" s="16" t="s">
@@ -3347,16 +3554,22 @@
       <c r="C15" s="17" t="s">
         <v>68</v>
       </c>
-      <c r="D15" s="17" t="s">
+      <c r="D15" s="20" t="s">
         <v>69</v>
       </c>
       <c r="E15" s="16" t="s">
         <v>70</v>
       </c>
-      <c r="F15" s="18"/>
+      <c r="F15" s="18" t="s">
+        <v>17</v>
+      </c>
       <c r="G15" s="18"/>
-      <c r="H15" s="15"/>
-      <c r="I15" s="15"/>
+      <c r="H15" s="15" t="s">
+        <v>17</v>
+      </c>
+      <c r="I15" s="15" t="s">
+        <v>17</v>
+      </c>
     </row>
     <row r="16" s="1" customFormat="1" ht="157.5" customHeight="1" spans="1:10">
       <c r="A16" s="16" t="s">
@@ -3368,18 +3581,24 @@
       <c r="C16" s="17" t="s">
         <v>73</v>
       </c>
-      <c r="D16" s="17" t="s">
+      <c r="D16" s="20" t="s">
         <v>74</v>
       </c>
       <c r="E16" s="17" t="s">
         <v>75</v>
       </c>
-      <c r="F16" s="18"/>
+      <c r="F16" s="18" t="s">
+        <v>17</v>
+      </c>
       <c r="G16" s="18"/>
-      <c r="H16" s="15"/>
-      <c r="I16" s="15"/>
-    </row>
-    <row r="17" s="1" customFormat="1" ht="78.75" customHeight="1" spans="1:9">
+      <c r="H16" s="15" t="s">
+        <v>17</v>
+      </c>
+      <c r="I16" s="15" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="17" s="1" customFormat="1" ht="189" spans="1:9">
       <c r="A17" s="16" t="s">
         <v>76</v>
       </c>
@@ -3389,333 +3608,407 @@
       <c r="C17" s="17" t="s">
         <v>78</v>
       </c>
-      <c r="D17" s="17" t="s">
+      <c r="D17" s="20" t="s">
         <v>79</v>
       </c>
       <c r="E17" s="17" t="s">
         <v>80</v>
       </c>
-      <c r="F17" s="18"/>
+      <c r="F17" s="18" t="s">
+        <v>81</v>
+      </c>
       <c r="G17" s="18"/>
-      <c r="H17" s="15"/>
-      <c r="I17" s="15"/>
+      <c r="H17" s="15" t="s">
+        <v>17</v>
+      </c>
+      <c r="I17" s="15" t="s">
+        <v>17</v>
+      </c>
     </row>
     <row r="18" s="1" customFormat="1" ht="15.75" customHeight="1" spans="1:9">
       <c r="A18" s="14" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="H18" s="15"/>
       <c r="I18" s="15"/>
     </row>
     <row r="19" s="1" customFormat="1" ht="78.75" customHeight="1" spans="1:9">
       <c r="A19" s="16" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="B19" s="16" t="s">
         <v>60</v>
       </c>
       <c r="C19" s="17" t="s">
-        <v>83</v>
-      </c>
-      <c r="D19" s="17" t="s">
         <v>84</v>
       </c>
+      <c r="D19" s="21" t="s">
+        <v>85</v>
+      </c>
       <c r="E19" s="16" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="F19" s="18"/>
       <c r="G19" s="18"/>
       <c r="H19" s="15"/>
       <c r="I19" s="15"/>
     </row>
-    <row r="20" s="1" customFormat="1" ht="94.5" customHeight="1" spans="1:9">
+    <row r="20" s="1" customFormat="1" ht="175.5" spans="1:9">
       <c r="A20" s="16" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="B20" s="16" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="C20" s="17" t="s">
-        <v>88</v>
-      </c>
-      <c r="D20" s="17" t="s">
         <v>89</v>
       </c>
+      <c r="D20" s="21" t="s">
+        <v>90</v>
+      </c>
       <c r="E20" s="17" t="s">
-        <v>90</v>
-      </c>
-      <c r="F20" s="18"/>
+        <v>91</v>
+      </c>
+      <c r="F20" s="18" t="s">
+        <v>92</v>
+      </c>
       <c r="G20" s="18"/>
-      <c r="H20" s="15"/>
+      <c r="H20" s="15" t="s">
+        <v>17</v>
+      </c>
       <c r="I20" s="15"/>
     </row>
-    <row r="21" s="1" customFormat="1" ht="63" customHeight="1" spans="1:9">
+    <row r="21" s="1" customFormat="1" ht="409.5" spans="1:9">
       <c r="A21" s="16" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="B21" s="16" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="C21" s="17" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="D21" s="17" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="E21" s="17" t="s">
-        <v>95</v>
-      </c>
-      <c r="F21" s="18"/>
+        <v>97</v>
+      </c>
+      <c r="F21" s="18" t="s">
+        <v>98</v>
+      </c>
       <c r="G21" s="18"/>
-      <c r="H21" s="15"/>
-      <c r="I21" s="15"/>
+      <c r="H21" s="15" t="s">
+        <v>17</v>
+      </c>
+      <c r="I21" s="15" t="s">
+        <v>17</v>
+      </c>
     </row>
     <row r="22" s="1" customFormat="1" ht="78.75" customHeight="1" spans="1:9">
       <c r="A22" s="16" t="s">
-        <v>96</v>
+        <v>99</v>
       </c>
       <c r="B22" s="16" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="C22" s="17" t="s">
-        <v>97</v>
-      </c>
-      <c r="D22" s="17" t="s">
-        <v>98</v>
+        <v>100</v>
+      </c>
+      <c r="D22" s="21" t="s">
+        <v>101</v>
       </c>
       <c r="E22" s="17" t="s">
-        <v>99</v>
-      </c>
-      <c r="F22" s="18"/>
+        <v>102</v>
+      </c>
+      <c r="F22" s="18" t="s">
+        <v>17</v>
+      </c>
       <c r="G22" s="18"/>
-      <c r="H22" s="15"/>
-      <c r="I22" s="15"/>
+      <c r="H22" s="15" t="s">
+        <v>17</v>
+      </c>
+      <c r="I22" s="15" t="s">
+        <v>17</v>
+      </c>
     </row>
     <row r="23" s="1" customFormat="1" ht="126" customHeight="1" spans="1:9">
       <c r="A23" s="17" t="s">
-        <v>100</v>
+        <v>103</v>
       </c>
       <c r="B23" s="17" t="s">
-        <v>101</v>
+        <v>104</v>
       </c>
       <c r="C23" s="17" t="s">
-        <v>102</v>
-      </c>
-      <c r="D23" s="17" t="s">
-        <v>103</v>
+        <v>105</v>
+      </c>
+      <c r="D23" s="21" t="s">
+        <v>106</v>
       </c>
       <c r="E23" s="17" t="s">
-        <v>104</v>
-      </c>
-      <c r="F23" s="18"/>
+        <v>107</v>
+      </c>
+      <c r="F23" s="18" t="s">
+        <v>17</v>
+      </c>
       <c r="G23" s="18"/>
-      <c r="H23" s="15"/>
-      <c r="I23" s="15"/>
+      <c r="H23" s="15" t="s">
+        <v>17</v>
+      </c>
+      <c r="I23" s="15" t="s">
+        <v>17</v>
+      </c>
     </row>
     <row r="24" s="1" customFormat="1" ht="126" customHeight="1" spans="1:9">
       <c r="A24" s="17" t="s">
-        <v>105</v>
+        <v>108</v>
       </c>
       <c r="B24" s="17" t="s">
-        <v>101</v>
+        <v>104</v>
       </c>
       <c r="C24" s="17" t="s">
-        <v>106</v>
-      </c>
-      <c r="D24" s="17" t="s">
-        <v>107</v>
+        <v>109</v>
+      </c>
+      <c r="D24" s="21" t="s">
+        <v>110</v>
       </c>
       <c r="E24" s="17" t="s">
-        <v>108</v>
-      </c>
-      <c r="F24" s="18"/>
+        <v>111</v>
+      </c>
+      <c r="F24" s="18" t="s">
+        <v>17</v>
+      </c>
       <c r="G24" s="18"/>
-      <c r="H24" s="15"/>
+      <c r="H24" s="15" t="s">
+        <v>17</v>
+      </c>
       <c r="I24" s="15"/>
     </row>
     <row r="25" s="1" customFormat="1" ht="173.25" customHeight="1" spans="1:9">
       <c r="A25" s="16" t="s">
-        <v>109</v>
+        <v>112</v>
       </c>
       <c r="B25" s="16" t="s">
-        <v>110</v>
+        <v>113</v>
       </c>
       <c r="C25" s="17" t="s">
-        <v>111</v>
-      </c>
-      <c r="D25" s="17" t="s">
-        <v>112</v>
+        <v>114</v>
+      </c>
+      <c r="D25" s="21" t="s">
+        <v>115</v>
       </c>
       <c r="E25" s="16" t="s">
-        <v>113</v>
-      </c>
-      <c r="F25" s="18"/>
+        <v>116</v>
+      </c>
+      <c r="F25" s="18" t="s">
+        <v>17</v>
+      </c>
       <c r="G25" s="18"/>
-      <c r="H25" s="15"/>
-      <c r="I25" s="15"/>
+      <c r="H25" s="15" t="s">
+        <v>17</v>
+      </c>
+      <c r="I25" s="15" t="s">
+        <v>17</v>
+      </c>
     </row>
     <row r="26" s="1" customFormat="1" ht="126" customHeight="1" spans="1:9">
       <c r="A26" s="16" t="s">
-        <v>114</v>
+        <v>117</v>
       </c>
       <c r="B26" s="16" t="s">
-        <v>110</v>
+        <v>113</v>
       </c>
       <c r="C26" s="17" t="s">
-        <v>115</v>
-      </c>
-      <c r="D26" s="17" t="s">
-        <v>116</v>
+        <v>118</v>
+      </c>
+      <c r="D26" s="21" t="s">
+        <v>119</v>
       </c>
       <c r="E26" s="16" t="s">
-        <v>117</v>
-      </c>
-      <c r="F26" s="18"/>
+        <v>120</v>
+      </c>
+      <c r="F26" s="18" t="s">
+        <v>17</v>
+      </c>
       <c r="G26" s="18"/>
-      <c r="H26" s="15"/>
-      <c r="I26" s="15"/>
+      <c r="H26" s="15" t="s">
+        <v>17</v>
+      </c>
+      <c r="I26" s="15" t="s">
+        <v>17</v>
+      </c>
     </row>
     <row r="27" s="1" customFormat="1" ht="220.5" customHeight="1" spans="1:9">
       <c r="A27" s="16" t="s">
-        <v>118</v>
+        <v>121</v>
       </c>
       <c r="B27" s="16" t="s">
-        <v>119</v>
+        <v>122</v>
       </c>
       <c r="C27" s="17" t="s">
-        <v>120</v>
-      </c>
-      <c r="D27" s="17" t="s">
-        <v>121</v>
+        <v>123</v>
+      </c>
+      <c r="D27" s="21" t="s">
+        <v>124</v>
       </c>
       <c r="E27" s="16" t="s">
-        <v>122</v>
-      </c>
-      <c r="F27" s="18"/>
+        <v>125</v>
+      </c>
+      <c r="F27" s="18" t="s">
+        <v>17</v>
+      </c>
       <c r="G27" s="18"/>
-      <c r="H27" s="15"/>
-      <c r="I27" s="15"/>
+      <c r="H27" s="15" t="s">
+        <v>17</v>
+      </c>
+      <c r="I27" s="15" t="s">
+        <v>17</v>
+      </c>
     </row>
     <row r="28" s="1" customFormat="1" ht="15.75" customHeight="1" spans="1:9">
       <c r="A28" s="14" t="s">
-        <v>123</v>
+        <v>126</v>
       </c>
       <c r="H28" s="15"/>
       <c r="I28" s="15"/>
     </row>
     <row r="29" s="1" customFormat="1" ht="63" customHeight="1" spans="1:9">
       <c r="A29" s="16" t="s">
-        <v>124</v>
+        <v>127</v>
       </c>
       <c r="B29" s="16" t="s">
-        <v>125</v>
+        <v>128</v>
       </c>
       <c r="C29" s="17" t="s">
-        <v>126</v>
-      </c>
-      <c r="D29" s="17" t="s">
-        <v>127</v>
+        <v>129</v>
+      </c>
+      <c r="D29" s="21" t="s">
+        <v>130</v>
       </c>
       <c r="E29" s="16" t="s">
-        <v>128</v>
-      </c>
-      <c r="F29" s="18"/>
+        <v>131</v>
+      </c>
+      <c r="F29" s="18" t="s">
+        <v>17</v>
+      </c>
       <c r="G29" s="18"/>
-      <c r="H29" s="15"/>
-      <c r="I29" s="15"/>
+      <c r="H29" s="15" t="s">
+        <v>17</v>
+      </c>
+      <c r="I29" s="15" t="s">
+        <v>17</v>
+      </c>
     </row>
     <row r="30" s="1" customFormat="1" ht="47.25" customHeight="1" spans="1:9">
       <c r="A30" s="16" t="s">
-        <v>129</v>
+        <v>132</v>
       </c>
       <c r="B30" s="16" t="s">
-        <v>130</v>
+        <v>133</v>
       </c>
       <c r="C30" s="17" t="s">
-        <v>131</v>
-      </c>
-      <c r="D30" s="17" t="s">
-        <v>132</v>
+        <v>134</v>
+      </c>
+      <c r="D30" s="21" t="s">
+        <v>135</v>
       </c>
       <c r="E30" s="17" t="s">
-        <v>133</v>
-      </c>
-      <c r="F30" s="18"/>
+        <v>136</v>
+      </c>
+      <c r="F30" s="18" t="s">
+        <v>17</v>
+      </c>
       <c r="G30" s="18"/>
-      <c r="H30" s="15"/>
-      <c r="I30" s="15"/>
+      <c r="H30" s="15" t="s">
+        <v>17</v>
+      </c>
+      <c r="I30" s="15" t="s">
+        <v>17</v>
+      </c>
     </row>
     <row r="31" s="1" customFormat="1" ht="15.75" customHeight="1" spans="1:9">
       <c r="A31" s="14" t="s">
-        <v>134</v>
+        <v>137</v>
       </c>
       <c r="H31" s="15"/>
       <c r="I31" s="15"/>
     </row>
     <row r="32" s="1" customFormat="1" ht="94.5" customHeight="1" spans="1:9">
       <c r="A32" s="16" t="s">
-        <v>135</v>
+        <v>138</v>
       </c>
       <c r="B32" s="16" t="s">
-        <v>136</v>
+        <v>139</v>
       </c>
       <c r="C32" s="17" t="s">
-        <v>137</v>
-      </c>
-      <c r="D32" s="17" t="s">
-        <v>138</v>
+        <v>140</v>
+      </c>
+      <c r="D32" s="21" t="s">
+        <v>141</v>
       </c>
       <c r="E32" s="16" t="s">
-        <v>139</v>
-      </c>
-      <c r="F32" s="18"/>
+        <v>142</v>
+      </c>
+      <c r="F32" s="18" t="s">
+        <v>143</v>
+      </c>
       <c r="G32" s="18"/>
-      <c r="H32" s="15"/>
-      <c r="I32" s="15"/>
-    </row>
-    <row r="33" s="1" customFormat="1" ht="94.5" customHeight="1" spans="1:9">
+      <c r="H32" s="15" t="s">
+        <v>17</v>
+      </c>
+      <c r="I32" s="15" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="33" s="1" customFormat="1" ht="108" spans="1:9">
       <c r="A33" s="16" t="s">
-        <v>140</v>
+        <v>144</v>
       </c>
       <c r="B33" s="16" t="s">
-        <v>110</v>
+        <v>113</v>
       </c>
       <c r="C33" s="17" t="s">
-        <v>141</v>
-      </c>
-      <c r="D33" s="17" t="s">
-        <v>142</v>
+        <v>145</v>
+      </c>
+      <c r="D33" s="21" t="s">
+        <v>146</v>
       </c>
       <c r="E33" s="17" t="s">
-        <v>143</v>
-      </c>
-      <c r="F33" s="18"/>
+        <v>147</v>
+      </c>
+      <c r="F33" s="18" t="s">
+        <v>148</v>
+      </c>
       <c r="G33" s="18"/>
-      <c r="H33" s="15"/>
-      <c r="I33" s="15"/>
+      <c r="H33" s="15" t="s">
+        <v>17</v>
+      </c>
+      <c r="I33" s="15" t="s">
+        <v>17</v>
+      </c>
     </row>
     <row r="34" s="1" customFormat="1" ht="15.75" customHeight="1" spans="1:9">
       <c r="A34" s="14" t="s">
-        <v>144</v>
+        <v>149</v>
       </c>
       <c r="H34" s="15"/>
       <c r="I34" s="15"/>
     </row>
     <row r="35" s="1" customFormat="1" ht="126" customHeight="1" spans="1:9">
       <c r="A35" s="16" t="s">
-        <v>145</v>
+        <v>150</v>
       </c>
       <c r="B35" s="16" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="C35" s="17" t="s">
-        <v>146</v>
+        <v>151</v>
       </c>
       <c r="D35" s="17" t="s">
-        <v>147</v>
+        <v>152</v>
       </c>
       <c r="E35" s="17" t="s">
-        <v>148</v>
+        <v>153</v>
       </c>
       <c r="F35" s="18"/>
       <c r="G35" s="18"/>
@@ -3724,19 +4017,19 @@
     </row>
     <row r="36" s="1" customFormat="1" ht="126" customHeight="1" spans="1:9">
       <c r="A36" s="16" t="s">
-        <v>149</v>
+        <v>154</v>
       </c>
       <c r="B36" s="16" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="C36" s="17" t="s">
-        <v>150</v>
+        <v>155</v>
       </c>
       <c r="D36" s="17" t="s">
-        <v>151</v>
+        <v>156</v>
       </c>
       <c r="E36" s="17" t="s">
-        <v>152</v>
+        <v>157</v>
       </c>
       <c r="F36" s="18"/>
       <c r="G36" s="18"/>
@@ -3745,19 +4038,19 @@
     </row>
     <row r="37" s="1" customFormat="1" ht="173.25" customHeight="1" spans="1:9">
       <c r="A37" s="16" t="s">
-        <v>153</v>
+        <v>158</v>
       </c>
       <c r="B37" s="16" t="s">
-        <v>154</v>
+        <v>159</v>
       </c>
       <c r="C37" s="17" t="s">
-        <v>155</v>
+        <v>160</v>
       </c>
       <c r="D37" s="17" t="s">
-        <v>156</v>
+        <v>161</v>
       </c>
       <c r="E37" s="17" t="s">
-        <v>157</v>
+        <v>162</v>
       </c>
       <c r="F37" s="18"/>
       <c r="G37" s="18"/>
@@ -3766,19 +4059,19 @@
     </row>
     <row r="38" s="1" customFormat="1" ht="141.75" customHeight="1" spans="1:9">
       <c r="A38" s="16" t="s">
-        <v>158</v>
+        <v>163</v>
       </c>
       <c r="B38" s="16" t="s">
-        <v>159</v>
+        <v>164</v>
       </c>
       <c r="C38" s="17" t="s">
-        <v>160</v>
+        <v>165</v>
       </c>
       <c r="D38" s="17" t="s">
-        <v>161</v>
+        <v>166</v>
       </c>
       <c r="E38" s="16" t="s">
-        <v>162</v>
+        <v>167</v>
       </c>
       <c r="F38" s="18"/>
       <c r="G38" s="18"/>
@@ -3787,19 +4080,19 @@
     </row>
     <row r="39" s="1" customFormat="1" ht="47.25" customHeight="1" spans="1:9">
       <c r="A39" s="16" t="s">
-        <v>163</v>
+        <v>168</v>
       </c>
       <c r="B39" s="16" t="s">
-        <v>164</v>
+        <v>169</v>
       </c>
       <c r="C39" s="17" t="s">
-        <v>165</v>
+        <v>170</v>
       </c>
       <c r="D39" s="16" t="s">
-        <v>166</v>
+        <v>171</v>
       </c>
       <c r="E39" s="16" t="s">
-        <v>167</v>
+        <v>172</v>
       </c>
       <c r="F39" s="18"/>
       <c r="G39" s="18"/>
@@ -3808,26 +4101,26 @@
     </row>
     <row r="40" s="1" customFormat="1" ht="15.75" customHeight="1" spans="1:9">
       <c r="A40" s="14" t="s">
-        <v>168</v>
+        <v>173</v>
       </c>
       <c r="H40" s="15"/>
       <c r="I40" s="15"/>
     </row>
     <row r="41" s="1" customFormat="1" ht="126" customHeight="1" spans="1:9">
       <c r="A41" s="16" t="s">
-        <v>169</v>
+        <v>174</v>
       </c>
       <c r="B41" s="16" t="s">
-        <v>170</v>
+        <v>175</v>
       </c>
       <c r="C41" s="17" t="s">
-        <v>171</v>
+        <v>176</v>
       </c>
       <c r="D41" s="17" t="s">
-        <v>172</v>
+        <v>177</v>
       </c>
       <c r="E41" s="17" t="s">
-        <v>173</v>
+        <v>178</v>
       </c>
       <c r="F41" s="18"/>
       <c r="G41" s="18"/>
@@ -3836,19 +4129,19 @@
     </row>
     <row r="42" s="1" customFormat="1" ht="110.25" customHeight="1" spans="1:9">
       <c r="A42" s="16" t="s">
-        <v>174</v>
+        <v>179</v>
       </c>
       <c r="B42" s="16" t="s">
-        <v>164</v>
+        <v>169</v>
       </c>
       <c r="C42" s="17" t="s">
-        <v>175</v>
+        <v>180</v>
       </c>
       <c r="D42" s="17" t="s">
-        <v>176</v>
+        <v>181</v>
       </c>
       <c r="E42" s="17" t="s">
-        <v>177</v>
+        <v>182</v>
       </c>
       <c r="F42" s="18"/>
       <c r="G42" s="18"/>
@@ -3857,19 +4150,19 @@
     </row>
     <row r="43" s="1" customFormat="1" ht="47.25" customHeight="1" spans="1:9">
       <c r="A43" s="16" t="s">
-        <v>178</v>
+        <v>183</v>
       </c>
       <c r="B43" s="16" t="s">
-        <v>164</v>
+        <v>169</v>
       </c>
       <c r="C43" s="17" t="s">
-        <v>179</v>
+        <v>184</v>
       </c>
       <c r="D43" s="16" t="s">
-        <v>166</v>
+        <v>171</v>
       </c>
       <c r="E43" s="16" t="s">
-        <v>180</v>
+        <v>185</v>
       </c>
       <c r="F43" s="18"/>
       <c r="G43" s="18"/>
@@ -3878,26 +4171,26 @@
     </row>
     <row r="44" s="1" customFormat="1" ht="15.75" customHeight="1" spans="1:9">
       <c r="A44" s="14" t="s">
-        <v>181</v>
+        <v>186</v>
       </c>
       <c r="H44" s="15"/>
       <c r="I44" s="15"/>
     </row>
     <row r="45" s="1" customFormat="1" ht="78.75" customHeight="1" spans="1:9">
       <c r="A45" s="16" t="s">
-        <v>182</v>
+        <v>187</v>
       </c>
       <c r="B45" s="16" t="s">
         <v>60</v>
       </c>
       <c r="C45" s="17" t="s">
-        <v>183</v>
+        <v>188</v>
       </c>
       <c r="D45" s="17" t="s">
-        <v>184</v>
+        <v>189</v>
       </c>
       <c r="E45" s="17" t="s">
-        <v>185</v>
+        <v>190</v>
       </c>
       <c r="F45" s="18"/>
       <c r="G45" s="18"/>
@@ -3906,19 +4199,19 @@
     </row>
     <row r="46" s="1" customFormat="1" ht="141.75" customHeight="1" spans="1:9">
       <c r="A46" s="16" t="s">
-        <v>186</v>
+        <v>191</v>
       </c>
       <c r="B46" s="16" t="s">
-        <v>164</v>
+        <v>169</v>
       </c>
       <c r="C46" s="17" t="s">
-        <v>187</v>
-      </c>
-      <c r="D46" s="17" t="s">
-        <v>188</v>
+        <v>192</v>
+      </c>
+      <c r="D46" s="21" t="s">
+        <v>193</v>
       </c>
       <c r="E46" s="17" t="s">
-        <v>189</v>
+        <v>194</v>
       </c>
       <c r="F46" s="18"/>
       <c r="G46" s="18"/>
@@ -3927,19 +4220,19 @@
     </row>
     <row r="47" s="1" customFormat="1" ht="47.25" customHeight="1" spans="1:9">
       <c r="A47" s="16" t="s">
-        <v>190</v>
+        <v>195</v>
       </c>
       <c r="B47" s="16" t="s">
-        <v>164</v>
+        <v>169</v>
       </c>
       <c r="C47" s="17" t="s">
-        <v>191</v>
+        <v>196</v>
       </c>
       <c r="D47" s="16" t="s">
-        <v>166</v>
+        <v>171</v>
       </c>
       <c r="E47" s="16" t="s">
-        <v>192</v>
+        <v>197</v>
       </c>
       <c r="F47" s="18"/>
       <c r="G47" s="18"/>
@@ -3948,26 +4241,26 @@
     </row>
     <row r="48" s="1" customFormat="1" ht="15.75" customHeight="1" spans="1:9">
       <c r="A48" s="14" t="s">
-        <v>193</v>
+        <v>198</v>
       </c>
       <c r="H48" s="15"/>
       <c r="I48" s="15"/>
     </row>
     <row r="49" s="1" customFormat="1" ht="94.5" customHeight="1" spans="1:9">
       <c r="A49" s="16" t="s">
-        <v>194</v>
+        <v>199</v>
       </c>
       <c r="B49" s="16" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="C49" s="17" t="s">
-        <v>195</v>
+        <v>200</v>
       </c>
       <c r="D49" s="17" t="s">
-        <v>196</v>
+        <v>201</v>
       </c>
       <c r="E49" s="17" t="s">
-        <v>197</v>
+        <v>202</v>
       </c>
       <c r="F49" s="18"/>
       <c r="G49" s="18"/>
@@ -3976,19 +4269,19 @@
     </row>
     <row r="50" s="1" customFormat="1" ht="126" customHeight="1" spans="1:9">
       <c r="A50" s="16" t="s">
-        <v>198</v>
+        <v>203</v>
       </c>
       <c r="B50" s="16" t="s">
-        <v>130</v>
+        <v>133</v>
       </c>
       <c r="C50" s="17" t="s">
-        <v>199</v>
+        <v>204</v>
       </c>
       <c r="D50" s="17" t="s">
-        <v>200</v>
+        <v>205</v>
       </c>
       <c r="E50" s="17" t="s">
-        <v>201</v>
+        <v>206</v>
       </c>
       <c r="F50" s="18"/>
       <c r="G50" s="18"/>
@@ -3997,26 +4290,26 @@
     </row>
     <row r="51" s="1" customFormat="1" ht="15.75" customHeight="1" spans="1:9">
       <c r="A51" s="14" t="s">
-        <v>202</v>
+        <v>207</v>
       </c>
       <c r="H51" s="15"/>
       <c r="I51" s="15"/>
     </row>
     <row r="52" s="1" customFormat="1" ht="63" customHeight="1" spans="1:9">
       <c r="A52" s="16" t="s">
-        <v>203</v>
+        <v>208</v>
       </c>
       <c r="B52" s="16" t="s">
-        <v>204</v>
+        <v>209</v>
       </c>
       <c r="C52" s="17" t="s">
-        <v>205</v>
+        <v>210</v>
       </c>
       <c r="D52" s="17" t="s">
-        <v>206</v>
+        <v>211</v>
       </c>
       <c r="E52" s="17" t="s">
-        <v>207</v>
+        <v>212</v>
       </c>
       <c r="F52" s="18"/>
       <c r="G52" s="18"/>
@@ -4025,26 +4318,26 @@
     </row>
     <row r="53" s="1" customFormat="1" ht="15.75" customHeight="1" spans="1:9">
       <c r="A53" s="14" t="s">
-        <v>208</v>
+        <v>213</v>
       </c>
       <c r="H53" s="15"/>
       <c r="I53" s="15"/>
     </row>
     <row r="54" s="1" customFormat="1" ht="220.5" customHeight="1" spans="1:9">
       <c r="A54" s="16" t="s">
-        <v>209</v>
+        <v>214</v>
       </c>
       <c r="B54" s="16" t="s">
-        <v>210</v>
+        <v>215</v>
       </c>
       <c r="C54" s="17" t="s">
-        <v>211</v>
+        <v>216</v>
       </c>
       <c r="D54" s="17" t="s">
-        <v>212</v>
+        <v>217</v>
       </c>
       <c r="E54" s="16" t="s">
-        <v>213</v>
+        <v>218</v>
       </c>
       <c r="F54" s="18"/>
       <c r="G54" s="18"/>
@@ -4053,26 +4346,26 @@
     </row>
     <row r="55" s="1" customFormat="1" ht="15.75" customHeight="1" spans="1:9">
       <c r="A55" s="14" t="s">
-        <v>214</v>
+        <v>219</v>
       </c>
       <c r="H55" s="15"/>
       <c r="I55" s="15"/>
     </row>
     <row r="56" s="1" customFormat="1" ht="78.75" customHeight="1" spans="1:9">
       <c r="A56" s="16" t="s">
-        <v>215</v>
+        <v>220</v>
       </c>
       <c r="B56" s="16" t="s">
-        <v>216</v>
+        <v>221</v>
       </c>
       <c r="C56" s="17" t="s">
-        <v>217</v>
+        <v>222</v>
       </c>
       <c r="D56" s="17" t="s">
-        <v>218</v>
+        <v>223</v>
       </c>
       <c r="E56" s="17" t="s">
-        <v>219</v>
+        <v>224</v>
       </c>
       <c r="F56" s="18"/>
       <c r="G56" s="18"/>
@@ -4081,19 +4374,19 @@
     </row>
     <row r="57" s="1" customFormat="1" ht="63" customHeight="1" spans="1:9">
       <c r="A57" s="16" t="s">
-        <v>220</v>
+        <v>225</v>
       </c>
       <c r="B57" s="16" t="s">
-        <v>221</v>
+        <v>226</v>
       </c>
       <c r="C57" s="17" t="s">
-        <v>222</v>
+        <v>227</v>
       </c>
       <c r="D57" s="17" t="s">
-        <v>223</v>
+        <v>228</v>
       </c>
       <c r="E57" s="17" t="s">
-        <v>224</v>
+        <v>229</v>
       </c>
       <c r="F57" s="18"/>
       <c r="G57" s="18"/>
@@ -4102,19 +4395,19 @@
     </row>
     <row r="58" s="1" customFormat="1" ht="47.25" customHeight="1" spans="1:9">
       <c r="A58" s="16" t="s">
-        <v>225</v>
+        <v>230</v>
       </c>
       <c r="B58" s="16" t="s">
-        <v>226</v>
+        <v>231</v>
       </c>
       <c r="C58" s="17" t="s">
-        <v>227</v>
+        <v>232</v>
       </c>
       <c r="D58" s="17" t="s">
-        <v>228</v>
+        <v>233</v>
       </c>
       <c r="E58" s="17" t="s">
-        <v>229</v>
+        <v>234</v>
       </c>
       <c r="F58" s="18"/>
       <c r="G58" s="18"/>
@@ -4123,19 +4416,19 @@
     </row>
     <row r="59" s="1" customFormat="1" ht="204.75" customHeight="1" spans="1:9">
       <c r="A59" s="16" t="s">
-        <v>230</v>
+        <v>235</v>
       </c>
       <c r="B59" s="16" t="s">
-        <v>231</v>
+        <v>236</v>
       </c>
       <c r="C59" s="17" t="s">
-        <v>232</v>
+        <v>237</v>
       </c>
       <c r="D59" s="17" t="s">
-        <v>233</v>
+        <v>238</v>
       </c>
       <c r="E59" s="17" t="s">
-        <v>234</v>
+        <v>239</v>
       </c>
       <c r="F59" s="18"/>
       <c r="G59" s="18"/>
@@ -4144,19 +4437,19 @@
     </row>
     <row r="60" s="1" customFormat="1" ht="267.75" customHeight="1" spans="1:9">
       <c r="A60" s="16" t="s">
-        <v>235</v>
+        <v>240</v>
       </c>
       <c r="B60" s="16" t="s">
-        <v>236</v>
+        <v>241</v>
       </c>
       <c r="C60" s="17" t="s">
-        <v>237</v>
+        <v>242</v>
       </c>
       <c r="D60" s="17" t="s">
         <v>24</v>
       </c>
       <c r="E60" s="17" t="s">
-        <v>238</v>
+        <v>243</v>
       </c>
       <c r="F60" s="18"/>
       <c r="G60" s="18"/>
@@ -4165,19 +4458,19 @@
     </row>
     <row r="61" s="1" customFormat="1" ht="78.75" customHeight="1" spans="1:9">
       <c r="A61" s="16" t="s">
-        <v>239</v>
+        <v>244</v>
       </c>
       <c r="B61" s="16" t="s">
-        <v>240</v>
+        <v>245</v>
       </c>
       <c r="C61" s="17" t="s">
-        <v>241</v>
+        <v>246</v>
       </c>
       <c r="D61" s="17" t="s">
-        <v>242</v>
+        <v>247</v>
       </c>
       <c r="E61" s="17" t="s">
-        <v>243</v>
+        <v>248</v>
       </c>
       <c r="F61" s="18"/>
       <c r="G61" s="18"/>
@@ -4186,19 +4479,19 @@
     </row>
     <row r="62" s="1" customFormat="1" ht="173.25" customHeight="1" spans="1:9">
       <c r="A62" s="16" t="s">
-        <v>244</v>
+        <v>249</v>
       </c>
       <c r="B62" s="16" t="s">
-        <v>110</v>
+        <v>113</v>
       </c>
       <c r="C62" s="17" t="s">
-        <v>245</v>
+        <v>250</v>
       </c>
       <c r="D62" s="17" t="s">
-        <v>246</v>
+        <v>251</v>
       </c>
       <c r="E62" s="16" t="s">
-        <v>247</v>
+        <v>252</v>
       </c>
       <c r="F62" s="18"/>
       <c r="G62" s="18"/>
@@ -4207,19 +4500,19 @@
     </row>
     <row r="63" s="1" customFormat="1" ht="157.5" customHeight="1" spans="1:9">
       <c r="A63" s="16" t="s">
-        <v>248</v>
+        <v>253</v>
       </c>
       <c r="B63" s="16" t="s">
-        <v>110</v>
+        <v>113</v>
       </c>
       <c r="C63" s="17" t="s">
-        <v>249</v>
+        <v>254</v>
       </c>
       <c r="D63" s="17" t="s">
-        <v>250</v>
+        <v>255</v>
       </c>
       <c r="E63" s="17" t="s">
-        <v>251</v>
+        <v>256</v>
       </c>
       <c r="F63" s="18"/>
       <c r="G63" s="18"/>
@@ -4228,26 +4521,26 @@
     </row>
     <row r="64" s="1" customFormat="1" ht="15.75" customHeight="1" spans="1:9">
       <c r="A64" s="14" t="s">
-        <v>252</v>
+        <v>257</v>
       </c>
       <c r="H64" s="15"/>
       <c r="I64" s="15"/>
     </row>
     <row r="65" s="1" customFormat="1" ht="126" customHeight="1" spans="1:9">
       <c r="A65" s="16" t="s">
-        <v>253</v>
+        <v>258</v>
       </c>
       <c r="B65" s="16" t="s">
-        <v>254</v>
+        <v>259</v>
       </c>
       <c r="C65" s="17" t="s">
-        <v>255</v>
+        <v>260</v>
       </c>
       <c r="D65" s="17" t="s">
-        <v>256</v>
+        <v>261</v>
       </c>
       <c r="E65" s="17" t="s">
-        <v>257</v>
+        <v>262</v>
       </c>
       <c r="F65" s="18"/>
       <c r="G65" s="18"/>
@@ -4256,19 +4549,19 @@
     </row>
     <row r="66" s="1" customFormat="1" ht="47.25" customHeight="1" spans="1:9">
       <c r="A66" s="16" t="s">
-        <v>258</v>
+        <v>263</v>
       </c>
       <c r="B66" s="16" t="s">
-        <v>259</v>
+        <v>264</v>
       </c>
       <c r="C66" s="17" t="s">
-        <v>260</v>
+        <v>265</v>
       </c>
       <c r="D66" s="17" t="s">
-        <v>261</v>
+        <v>266</v>
       </c>
       <c r="E66" s="16" t="s">
-        <v>262</v>
+        <v>267</v>
       </c>
       <c r="F66" s="18"/>
       <c r="G66" s="18"/>
@@ -4277,26 +4570,26 @@
     </row>
     <row r="67" s="1" customFormat="1" ht="15.75" customHeight="1" spans="1:9">
       <c r="A67" s="14" t="s">
-        <v>263</v>
+        <v>268</v>
       </c>
       <c r="H67" s="15"/>
       <c r="I67" s="15"/>
     </row>
     <row r="68" s="1" customFormat="1" ht="94.5" customHeight="1" spans="1:9">
       <c r="A68" s="16" t="s">
-        <v>264</v>
+        <v>269</v>
       </c>
       <c r="B68" s="16" t="s">
-        <v>254</v>
+        <v>259</v>
       </c>
       <c r="C68" s="17" t="s">
-        <v>265</v>
+        <v>270</v>
       </c>
       <c r="D68" s="17" t="s">
-        <v>266</v>
+        <v>271</v>
       </c>
       <c r="E68" s="16" t="s">
-        <v>267</v>
+        <v>272</v>
       </c>
       <c r="F68" s="18"/>
       <c r="G68" s="18"/>
@@ -4305,19 +4598,19 @@
     </row>
     <row r="69" s="1" customFormat="1" ht="47.25" customHeight="1" spans="1:9">
       <c r="A69" s="16" t="s">
-        <v>268</v>
+        <v>273</v>
       </c>
       <c r="B69" s="16" t="s">
-        <v>269</v>
+        <v>274</v>
       </c>
       <c r="C69" s="17" t="s">
-        <v>270</v>
+        <v>275</v>
       </c>
       <c r="D69" s="17" t="s">
-        <v>271</v>
+        <v>276</v>
       </c>
       <c r="E69" s="16" t="s">
-        <v>272</v>
+        <v>277</v>
       </c>
       <c r="F69" s="18"/>
       <c r="G69" s="18"/>
@@ -4326,26 +4619,26 @@
     </row>
     <row r="70" s="1" customFormat="1" ht="15.75" customHeight="1" spans="1:9">
       <c r="A70" s="14" t="s">
-        <v>273</v>
+        <v>278</v>
       </c>
       <c r="H70" s="15"/>
       <c r="I70" s="15"/>
     </row>
     <row r="71" s="1" customFormat="1" ht="126" customHeight="1" spans="1:9">
       <c r="A71" s="16" t="s">
-        <v>274</v>
+        <v>279</v>
       </c>
       <c r="B71" s="16" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="C71" s="17" t="s">
-        <v>275</v>
+        <v>280</v>
       </c>
       <c r="D71" s="17" t="s">
-        <v>276</v>
+        <v>281</v>
       </c>
       <c r="E71" s="17" t="s">
-        <v>277</v>
+        <v>282</v>
       </c>
       <c r="F71" s="18"/>
       <c r="G71" s="18"/>
@@ -4354,19 +4647,19 @@
     </row>
     <row r="72" s="1" customFormat="1" ht="78.75" customHeight="1" spans="1:9">
       <c r="A72" s="17" t="s">
-        <v>278</v>
+        <v>283</v>
       </c>
       <c r="B72" s="17" t="s">
-        <v>279</v>
+        <v>284</v>
       </c>
       <c r="C72" s="17" t="s">
-        <v>280</v>
+        <v>285</v>
       </c>
       <c r="D72" s="17" t="s">
-        <v>138</v>
+        <v>141</v>
       </c>
       <c r="E72" s="17" t="s">
-        <v>281</v>
+        <v>286</v>
       </c>
       <c r="F72" s="18"/>
       <c r="G72" s="18"/>
@@ -4375,19 +4668,19 @@
     </row>
     <row r="73" s="1" customFormat="1" ht="315" customHeight="1" spans="1:9">
       <c r="A73" s="16" t="s">
-        <v>282</v>
+        <v>287</v>
       </c>
       <c r="B73" s="16" t="s">
-        <v>283</v>
+        <v>288</v>
       </c>
       <c r="C73" s="17" t="s">
-        <v>284</v>
+        <v>289</v>
       </c>
       <c r="D73" s="17" t="s">
-        <v>285</v>
+        <v>290</v>
       </c>
       <c r="E73" s="16" t="s">
-        <v>286</v>
+        <v>291</v>
       </c>
       <c r="F73" s="18"/>
       <c r="G73" s="18"/>
@@ -4396,19 +4689,19 @@
     </row>
     <row r="74" s="1" customFormat="1" ht="63" customHeight="1" spans="1:9">
       <c r="A74" s="16" t="s">
-        <v>287</v>
+        <v>292</v>
       </c>
       <c r="B74" s="16" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="C74" s="17" t="s">
-        <v>288</v>
+        <v>293</v>
       </c>
       <c r="D74" s="17" t="s">
-        <v>289</v>
+        <v>294</v>
       </c>
       <c r="E74" s="16" t="s">
-        <v>290</v>
+        <v>295</v>
       </c>
       <c r="F74" s="18"/>
       <c r="G74" s="18"/>
@@ -4417,19 +4710,19 @@
     </row>
     <row r="75" s="1" customFormat="1" ht="78.75" customHeight="1" spans="1:9">
       <c r="A75" s="16" t="s">
-        <v>291</v>
+        <v>296</v>
       </c>
       <c r="B75" s="16" t="s">
-        <v>292</v>
+        <v>297</v>
       </c>
       <c r="C75" s="17" t="s">
-        <v>293</v>
+        <v>298</v>
       </c>
       <c r="D75" s="17" t="s">
-        <v>294</v>
+        <v>299</v>
       </c>
       <c r="E75" s="16" t="s">
-        <v>295</v>
+        <v>300</v>
       </c>
       <c r="F75" s="18"/>
       <c r="G75" s="18"/>
@@ -4438,54 +4731,60 @@
     </row>
     <row r="76" s="1" customFormat="1" ht="15.75" customHeight="1" spans="1:9">
       <c r="A76" s="14" t="s">
-        <v>296</v>
+        <v>301</v>
       </c>
       <c r="H76" s="15"/>
       <c r="I76" s="15"/>
     </row>
     <row r="77" s="1" customFormat="1" ht="157.5" customHeight="1" spans="1:9">
       <c r="A77" s="16" t="s">
-        <v>297</v>
+        <v>302</v>
       </c>
       <c r="B77" s="16" t="s">
-        <v>298</v>
+        <v>303</v>
       </c>
       <c r="C77" s="17" t="s">
-        <v>299</v>
-      </c>
-      <c r="D77" s="17" t="s">
-        <v>300</v>
+        <v>304</v>
+      </c>
+      <c r="D77" s="21" t="s">
+        <v>305</v>
       </c>
       <c r="E77" s="17" t="s">
-        <v>301</v>
-      </c>
-      <c r="F77" s="18"/>
+        <v>306</v>
+      </c>
+      <c r="F77" s="18" t="s">
+        <v>307</v>
+      </c>
       <c r="G77" s="18"/>
-      <c r="H77" s="15"/>
-      <c r="I77" s="15"/>
+      <c r="H77" s="15" t="s">
+        <v>17</v>
+      </c>
+      <c r="I77" s="15" t="s">
+        <v>17</v>
+      </c>
     </row>
     <row r="78" s="1" customFormat="1" ht="15.75" customHeight="1" spans="1:9">
       <c r="A78" s="14" t="s">
-        <v>302</v>
+        <v>308</v>
       </c>
       <c r="H78" s="15"/>
       <c r="I78" s="15"/>
     </row>
     <row r="79" s="1" customFormat="1" ht="94.5" customHeight="1" spans="1:9">
       <c r="A79" s="16" t="s">
-        <v>303</v>
+        <v>309</v>
       </c>
       <c r="B79" s="16" t="s">
-        <v>304</v>
+        <v>310</v>
       </c>
       <c r="C79" s="17" t="s">
-        <v>305</v>
-      </c>
-      <c r="D79" s="17" t="s">
+        <v>311</v>
+      </c>
+      <c r="D79" s="21" t="s">
         <v>40</v>
       </c>
       <c r="E79" s="16" t="s">
-        <v>306</v>
+        <v>312</v>
       </c>
       <c r="F79" s="18"/>
       <c r="G79" s="18"/>
@@ -4494,19 +4793,19 @@
     </row>
     <row r="80" s="1" customFormat="1" ht="173.25" customHeight="1" spans="1:9">
       <c r="A80" s="16" t="s">
-        <v>307</v>
+        <v>313</v>
       </c>
       <c r="B80" s="16" t="s">
-        <v>308</v>
+        <v>314</v>
       </c>
       <c r="C80" s="17" t="s">
-        <v>309</v>
+        <v>315</v>
       </c>
       <c r="D80" s="17" t="s">
-        <v>310</v>
+        <v>316</v>
       </c>
       <c r="E80" s="17" t="s">
-        <v>311</v>
+        <v>317</v>
       </c>
       <c r="F80" s="18"/>
       <c r="G80" s="18"/>
@@ -4515,19 +4814,19 @@
     </row>
     <row r="81" s="1" customFormat="1" ht="157.5" customHeight="1" spans="1:9">
       <c r="A81" s="16" t="s">
-        <v>312</v>
+        <v>318</v>
       </c>
       <c r="B81" s="16" t="s">
-        <v>308</v>
+        <v>314</v>
       </c>
       <c r="C81" s="17" t="s">
-        <v>313</v>
+        <v>319</v>
       </c>
       <c r="D81" s="17" t="s">
-        <v>314</v>
+        <v>320</v>
       </c>
       <c r="E81" s="17" t="s">
-        <v>315</v>
+        <v>321</v>
       </c>
       <c r="F81" s="18"/>
       <c r="G81" s="18"/>
@@ -4536,19 +4835,19 @@
     </row>
     <row r="82" s="1" customFormat="1" ht="220.5" customHeight="1" spans="1:9">
       <c r="A82" s="16" t="s">
-        <v>316</v>
+        <v>322</v>
       </c>
       <c r="B82" s="16" t="s">
-        <v>308</v>
+        <v>314</v>
       </c>
       <c r="C82" s="17" t="s">
-        <v>317</v>
+        <v>323</v>
       </c>
       <c r="D82" s="17" t="s">
-        <v>318</v>
+        <v>324</v>
       </c>
       <c r="E82" s="17" t="s">
-        <v>319</v>
+        <v>325</v>
       </c>
       <c r="F82" s="18"/>
       <c r="G82" s="18"/>
@@ -4557,10 +4856,10 @@
     </row>
     <row r="83" s="1" customFormat="1" ht="126" customHeight="1" spans="1:9">
       <c r="A83" s="16" t="s">
-        <v>320</v>
+        <v>326</v>
       </c>
       <c r="B83" s="16" t="s">
-        <v>321</v>
+        <v>327</v>
       </c>
       <c r="C83" s="17" t="s">
         <v>50</v>
@@ -4569,7 +4868,7 @@
         <v>51</v>
       </c>
       <c r="E83" s="17" t="s">
-        <v>322</v>
+        <v>328</v>
       </c>
       <c r="F83" s="18"/>
       <c r="G83" s="18"/>
@@ -4578,19 +4877,19 @@
     </row>
     <row r="84" s="1" customFormat="1" ht="78.75" customHeight="1" spans="1:9">
       <c r="A84" s="16" t="s">
-        <v>323</v>
+        <v>329</v>
       </c>
       <c r="B84" s="16" t="s">
-        <v>324</v>
+        <v>330</v>
       </c>
       <c r="C84" s="17" t="s">
-        <v>325</v>
+        <v>331</v>
       </c>
       <c r="D84" s="17" t="s">
-        <v>326</v>
+        <v>332</v>
       </c>
       <c r="E84" s="17" t="s">
-        <v>327</v>
+        <v>333</v>
       </c>
       <c r="F84" s="18"/>
       <c r="G84" s="18"/>
@@ -4599,19 +4898,19 @@
     </row>
     <row r="85" s="1" customFormat="1" ht="78.75" customHeight="1" spans="1:9">
       <c r="A85" s="16" t="s">
-        <v>328</v>
+        <v>334</v>
       </c>
       <c r="B85" s="16" t="s">
-        <v>324</v>
+        <v>330</v>
       </c>
       <c r="C85" s="17" t="s">
-        <v>329</v>
+        <v>335</v>
       </c>
       <c r="D85" s="17" t="s">
-        <v>330</v>
+        <v>336</v>
       </c>
       <c r="E85" s="17" t="s">
-        <v>331</v>
+        <v>337</v>
       </c>
       <c r="F85" s="18"/>
       <c r="G85" s="18"/>
@@ -4620,19 +4919,19 @@
     </row>
     <row r="86" s="1" customFormat="1" ht="78.75" customHeight="1" spans="1:9">
       <c r="A86" s="16" t="s">
-        <v>332</v>
+        <v>338</v>
       </c>
       <c r="B86" s="16" t="s">
-        <v>333</v>
+        <v>339</v>
       </c>
       <c r="C86" s="17" t="s">
-        <v>334</v>
+        <v>340</v>
       </c>
       <c r="D86" s="17" t="s">
-        <v>335</v>
+        <v>341</v>
       </c>
       <c r="E86" s="17" t="s">
-        <v>336</v>
+        <v>342</v>
       </c>
       <c r="F86" s="18"/>
       <c r="G86" s="18"/>
@@ -4641,19 +4940,19 @@
     </row>
     <row r="87" s="1" customFormat="1" ht="78.75" customHeight="1" spans="1:9">
       <c r="A87" s="16" t="s">
-        <v>337</v>
+        <v>343</v>
       </c>
       <c r="B87" s="16" t="s">
-        <v>333</v>
+        <v>339</v>
       </c>
       <c r="C87" s="17" t="s">
-        <v>338</v>
+        <v>344</v>
       </c>
       <c r="D87" s="17" t="s">
-        <v>339</v>
+        <v>345</v>
       </c>
       <c r="E87" s="17" t="s">
-        <v>340</v>
+        <v>346</v>
       </c>
       <c r="F87" s="18"/>
       <c r="G87" s="18"/>
@@ -4662,26 +4961,26 @@
     </row>
     <row r="88" s="1" customFormat="1" ht="15.75" customHeight="1" spans="1:9">
       <c r="A88" s="14" t="s">
-        <v>341</v>
+        <v>347</v>
       </c>
       <c r="H88" s="15"/>
       <c r="I88" s="15"/>
     </row>
     <row r="89" s="1" customFormat="1" ht="78.75" customHeight="1" spans="1:9">
       <c r="A89" s="16" t="s">
-        <v>342</v>
+        <v>348</v>
       </c>
       <c r="B89" s="16" t="s">
-        <v>343</v>
+        <v>349</v>
       </c>
       <c r="C89" s="17" t="s">
-        <v>344</v>
-      </c>
-      <c r="D89" s="17" t="s">
+        <v>350</v>
+      </c>
+      <c r="D89" s="20" t="s">
         <v>79</v>
       </c>
       <c r="E89" s="16" t="s">
-        <v>345</v>
+        <v>351</v>
       </c>
       <c r="F89" s="18"/>
       <c r="G89" s="18"/>
@@ -4690,19 +4989,19 @@
     </row>
     <row r="90" s="1" customFormat="1" ht="173.25" customHeight="1" spans="1:9">
       <c r="A90" s="16" t="s">
-        <v>346</v>
+        <v>352</v>
       </c>
       <c r="B90" s="16" t="s">
-        <v>308</v>
+        <v>314</v>
       </c>
       <c r="C90" s="17" t="s">
-        <v>347</v>
+        <v>353</v>
       </c>
       <c r="D90" s="17" t="s">
-        <v>348</v>
+        <v>354</v>
       </c>
       <c r="E90" s="17" t="s">
-        <v>311</v>
+        <v>317</v>
       </c>
       <c r="F90" s="18"/>
       <c r="G90" s="18"/>
@@ -4711,19 +5010,19 @@
     </row>
     <row r="91" s="1" customFormat="1" ht="94.5" customHeight="1" spans="1:9">
       <c r="A91" s="16" t="s">
-        <v>349</v>
+        <v>355</v>
       </c>
       <c r="B91" s="16" t="s">
-        <v>308</v>
+        <v>314</v>
       </c>
       <c r="C91" s="17" t="s">
-        <v>350</v>
+        <v>356</v>
       </c>
       <c r="D91" s="17" t="s">
-        <v>351</v>
+        <v>357</v>
       </c>
       <c r="E91" s="17" t="s">
-        <v>352</v>
+        <v>358</v>
       </c>
       <c r="F91" s="18"/>
       <c r="G91" s="18"/>
@@ -4732,19 +5031,19 @@
     </row>
     <row r="92" s="1" customFormat="1" ht="220.5" customHeight="1" spans="1:9">
       <c r="A92" s="16" t="s">
-        <v>353</v>
+        <v>359</v>
       </c>
       <c r="B92" s="16" t="s">
-        <v>308</v>
+        <v>314</v>
       </c>
       <c r="C92" s="17" t="s">
-        <v>354</v>
+        <v>360</v>
       </c>
       <c r="D92" s="17" t="s">
-        <v>355</v>
+        <v>361</v>
       </c>
       <c r="E92" s="17" t="s">
-        <v>319</v>
+        <v>325</v>
       </c>
       <c r="F92" s="18"/>
       <c r="G92" s="18"/>
@@ -4753,19 +5052,19 @@
     </row>
     <row r="93" s="1" customFormat="1" ht="141.75" customHeight="1" spans="1:9">
       <c r="A93" s="16" t="s">
-        <v>356</v>
+        <v>362</v>
       </c>
       <c r="B93" s="16" t="s">
-        <v>357</v>
+        <v>363</v>
       </c>
       <c r="C93" s="17" t="s">
-        <v>358</v>
+        <v>364</v>
       </c>
       <c r="D93" s="17" t="s">
-        <v>359</v>
+        <v>365</v>
       </c>
       <c r="E93" s="17" t="s">
-        <v>360</v>
+        <v>366</v>
       </c>
       <c r="F93" s="18"/>
       <c r="G93" s="18"/>
@@ -4774,19 +5073,19 @@
     </row>
     <row r="94" s="1" customFormat="1" ht="173.25" customHeight="1" spans="1:9">
       <c r="A94" s="16" t="s">
-        <v>361</v>
+        <v>367</v>
       </c>
       <c r="B94" s="16" t="s">
-        <v>308</v>
+        <v>314</v>
       </c>
       <c r="C94" s="17" t="s">
-        <v>362</v>
+        <v>368</v>
       </c>
       <c r="D94" s="17" t="s">
-        <v>363</v>
+        <v>369</v>
       </c>
       <c r="E94" s="17" t="s">
-        <v>364</v>
+        <v>370</v>
       </c>
       <c r="F94" s="18"/>
       <c r="G94" s="18"/>
@@ -4795,19 +5094,19 @@
     </row>
     <row r="95" s="1" customFormat="1" ht="173.25" customHeight="1" spans="1:9">
       <c r="A95" s="16" t="s">
-        <v>365</v>
+        <v>371</v>
       </c>
       <c r="B95" s="16" t="s">
-        <v>308</v>
+        <v>314</v>
       </c>
       <c r="C95" s="17" t="s">
-        <v>366</v>
+        <v>372</v>
       </c>
       <c r="D95" s="17" t="s">
-        <v>367</v>
+        <v>373</v>
       </c>
       <c r="E95" s="17" t="s">
-        <v>368</v>
+        <v>374</v>
       </c>
       <c r="F95" s="18"/>
       <c r="G95" s="18"/>
@@ -4816,19 +5115,19 @@
     </row>
     <row r="96" s="1" customFormat="1" ht="126" customHeight="1" spans="1:9">
       <c r="A96" s="16" t="s">
-        <v>369</v>
+        <v>375</v>
       </c>
       <c r="B96" s="16" t="s">
-        <v>357</v>
+        <v>363</v>
       </c>
       <c r="C96" s="17" t="s">
-        <v>370</v>
+        <v>376</v>
       </c>
       <c r="D96" s="17" t="s">
-        <v>371</v>
+        <v>377</v>
       </c>
       <c r="E96" s="17" t="s">
-        <v>372</v>
+        <v>378</v>
       </c>
       <c r="F96" s="18"/>
       <c r="G96" s="18"/>
@@ -4837,19 +5136,19 @@
     </row>
     <row r="97" s="1" customFormat="1" ht="78.75" customHeight="1" spans="1:9">
       <c r="A97" s="16" t="s">
-        <v>373</v>
+        <v>379</v>
       </c>
       <c r="B97" s="16" t="s">
-        <v>324</v>
+        <v>330</v>
       </c>
       <c r="C97" s="17" t="s">
-        <v>374</v>
+        <v>380</v>
       </c>
       <c r="D97" s="17" t="s">
-        <v>375</v>
+        <v>381</v>
       </c>
       <c r="E97" s="17" t="s">
-        <v>340</v>
+        <v>346</v>
       </c>
       <c r="F97" s="18"/>
       <c r="G97" s="18"/>
@@ -4858,19 +5157,19 @@
     </row>
     <row r="98" s="1" customFormat="1" ht="78.75" customHeight="1" spans="1:9">
       <c r="A98" s="16" t="s">
-        <v>376</v>
+        <v>382</v>
       </c>
       <c r="B98" s="16" t="s">
-        <v>377</v>
+        <v>383</v>
       </c>
       <c r="C98" s="17" t="s">
-        <v>378</v>
+        <v>384</v>
       </c>
       <c r="D98" s="17" t="s">
-        <v>379</v>
+        <v>385</v>
       </c>
       <c r="E98" s="17" t="s">
-        <v>380</v>
+        <v>386</v>
       </c>
       <c r="F98" s="18"/>
       <c r="G98" s="18"/>
@@ -4879,19 +5178,19 @@
     </row>
     <row r="99" s="1" customFormat="1" ht="78.75" customHeight="1" spans="1:9">
       <c r="A99" s="16" t="s">
-        <v>381</v>
+        <v>387</v>
       </c>
       <c r="B99" s="16" t="s">
-        <v>382</v>
+        <v>388</v>
       </c>
       <c r="C99" s="17" t="s">
-        <v>383</v>
+        <v>389</v>
       </c>
       <c r="D99" s="17" t="s">
-        <v>384</v>
+        <v>390</v>
       </c>
       <c r="E99" s="17" t="s">
-        <v>385</v>
+        <v>391</v>
       </c>
       <c r="F99" s="18"/>
       <c r="G99" s="18"/>
@@ -4900,26 +5199,26 @@
     </row>
     <row r="100" s="1" customFormat="1" ht="15.75" customHeight="1" spans="1:9">
       <c r="A100" s="14" t="s">
-        <v>386</v>
+        <v>392</v>
       </c>
       <c r="H100" s="15"/>
       <c r="I100" s="15"/>
     </row>
     <row r="101" s="1" customFormat="1" ht="78.75" customHeight="1" spans="1:9">
       <c r="A101" s="16" t="s">
-        <v>387</v>
+        <v>393</v>
       </c>
       <c r="B101" s="16" t="s">
-        <v>388</v>
+        <v>394</v>
       </c>
       <c r="C101" s="17" t="s">
-        <v>389</v>
+        <v>395</v>
       </c>
       <c r="D101" s="17" t="s">
-        <v>390</v>
+        <v>396</v>
       </c>
       <c r="E101" s="17" t="s">
-        <v>391</v>
+        <v>397</v>
       </c>
       <c r="F101" s="18"/>
       <c r="G101" s="18"/>
@@ -4928,19 +5227,19 @@
     </row>
     <row r="102" s="1" customFormat="1" ht="78.75" customHeight="1" spans="1:9">
       <c r="A102" s="16" t="s">
-        <v>392</v>
+        <v>398</v>
       </c>
       <c r="B102" s="16" t="s">
-        <v>393</v>
+        <v>399</v>
       </c>
       <c r="C102" s="17" t="s">
-        <v>394</v>
-      </c>
-      <c r="D102" s="17" t="s">
-        <v>395</v>
+        <v>400</v>
+      </c>
+      <c r="D102" s="20" t="s">
+        <v>401</v>
       </c>
       <c r="E102" s="17" t="s">
-        <v>396</v>
+        <v>402</v>
       </c>
       <c r="F102" s="18"/>
       <c r="G102" s="18"/>
@@ -4949,19 +5248,19 @@
     </row>
     <row r="103" s="1" customFormat="1" ht="78.75" customHeight="1" spans="1:9">
       <c r="A103" s="16" t="s">
-        <v>397</v>
+        <v>403</v>
       </c>
       <c r="B103" s="16" t="s">
-        <v>388</v>
+        <v>394</v>
       </c>
       <c r="C103" s="17" t="s">
-        <v>398</v>
-      </c>
-      <c r="D103" s="17" t="s">
-        <v>399</v>
+        <v>404</v>
+      </c>
+      <c r="D103" s="20" t="s">
+        <v>405</v>
       </c>
       <c r="E103" s="17" t="s">
-        <v>400</v>
+        <v>406</v>
       </c>
       <c r="F103" s="18"/>
       <c r="G103" s="18"/>
@@ -4970,19 +5269,19 @@
     </row>
     <row r="104" s="1" customFormat="1" ht="78.75" customHeight="1" spans="1:9">
       <c r="A104" s="16" t="s">
-        <v>401</v>
+        <v>407</v>
       </c>
       <c r="B104" s="16" t="s">
-        <v>402</v>
+        <v>408</v>
       </c>
       <c r="C104" s="17" t="s">
-        <v>241</v>
+        <v>246</v>
       </c>
       <c r="D104" s="17" t="s">
-        <v>242</v>
+        <v>247</v>
       </c>
       <c r="E104" s="16" t="s">
-        <v>403</v>
+        <v>409</v>
       </c>
       <c r="F104" s="18"/>
       <c r="G104" s="18"/>
@@ -4991,26 +5290,26 @@
     </row>
     <row r="105" s="1" customFormat="1" ht="15.75" customHeight="1" spans="1:9">
       <c r="A105" s="14" t="s">
-        <v>404</v>
+        <v>410</v>
       </c>
       <c r="H105" s="15"/>
       <c r="I105" s="15"/>
     </row>
     <row r="106" s="1" customFormat="1" ht="94.5" customHeight="1" spans="1:9">
       <c r="A106" s="16" t="s">
-        <v>405</v>
+        <v>411</v>
       </c>
       <c r="B106" s="16" t="s">
-        <v>406</v>
+        <v>412</v>
       </c>
       <c r="C106" s="17" t="s">
-        <v>141</v>
+        <v>145</v>
       </c>
       <c r="D106" s="17" t="s">
-        <v>142</v>
+        <v>146</v>
       </c>
       <c r="E106" s="16" t="s">
-        <v>407</v>
+        <v>413</v>
       </c>
       <c r="F106" s="18"/>
       <c r="G106" s="18"/>
@@ -5019,19 +5318,19 @@
     </row>
     <row r="107" s="1" customFormat="1" ht="252" customHeight="1" spans="1:9">
       <c r="A107" s="16" t="s">
-        <v>408</v>
+        <v>414</v>
       </c>
       <c r="B107" s="16" t="s">
-        <v>409</v>
+        <v>415</v>
       </c>
       <c r="C107" s="17" t="s">
-        <v>410</v>
+        <v>416</v>
       </c>
       <c r="D107" s="17" t="s">
-        <v>411</v>
+        <v>417</v>
       </c>
       <c r="E107" s="17" t="s">
-        <v>319</v>
+        <v>325</v>
       </c>
       <c r="F107" s="18"/>
       <c r="G107" s="18"/>
@@ -5040,19 +5339,19 @@
     </row>
     <row r="108" s="1" customFormat="1" ht="236.25" customHeight="1" spans="1:9">
       <c r="A108" s="16" t="s">
-        <v>412</v>
+        <v>418</v>
       </c>
       <c r="B108" s="16" t="s">
-        <v>413</v>
+        <v>419</v>
       </c>
       <c r="C108" s="17" t="s">
-        <v>414</v>
+        <v>420</v>
       </c>
       <c r="D108" s="17" t="s">
-        <v>415</v>
+        <v>421</v>
       </c>
       <c r="E108" s="17" t="s">
-        <v>416</v>
+        <v>422</v>
       </c>
       <c r="F108" s="18"/>
       <c r="G108" s="18"/>
@@ -5061,19 +5360,19 @@
     </row>
     <row r="109" s="1" customFormat="1" ht="141.75" customHeight="1" spans="1:9">
       <c r="A109" s="16" t="s">
-        <v>417</v>
+        <v>423</v>
       </c>
       <c r="B109" s="16" t="s">
-        <v>418</v>
+        <v>424</v>
       </c>
       <c r="C109" s="17" t="s">
-        <v>419</v>
+        <v>425</v>
       </c>
       <c r="D109" s="17" t="s">
-        <v>420</v>
+        <v>426</v>
       </c>
       <c r="E109" s="17" t="s">
-        <v>421</v>
+        <v>427</v>
       </c>
       <c r="F109" s="18"/>
       <c r="G109" s="18"/>
@@ -5082,19 +5381,19 @@
     </row>
     <row r="110" s="1" customFormat="1" ht="78.75" customHeight="1" spans="1:9">
       <c r="A110" s="16" t="s">
-        <v>422</v>
+        <v>428</v>
       </c>
       <c r="B110" s="16" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="C110" s="17" t="s">
-        <v>423</v>
+        <v>429</v>
       </c>
       <c r="D110" s="17" t="s">
-        <v>424</v>
+        <v>430</v>
       </c>
       <c r="E110" s="17" t="s">
-        <v>425</v>
+        <v>431</v>
       </c>
       <c r="F110" s="18"/>
       <c r="G110" s="18"/>
@@ -5103,19 +5402,19 @@
     </row>
     <row r="111" s="1" customFormat="1" ht="78.75" customHeight="1" spans="1:9">
       <c r="A111" s="16" t="s">
-        <v>426</v>
+        <v>432</v>
       </c>
       <c r="B111" s="16" t="s">
-        <v>427</v>
+        <v>433</v>
       </c>
       <c r="C111" s="17" t="s">
-        <v>428</v>
+        <v>434</v>
       </c>
       <c r="D111" s="17" t="s">
-        <v>429</v>
+        <v>435</v>
       </c>
       <c r="E111" s="17" t="s">
-        <v>430</v>
+        <v>436</v>
       </c>
       <c r="F111" s="18"/>
       <c r="G111" s="18"/>
@@ -5124,19 +5423,19 @@
     </row>
     <row r="112" s="1" customFormat="1" ht="78.75" customHeight="1" spans="1:9">
       <c r="A112" s="16" t="s">
-        <v>431</v>
+        <v>437</v>
       </c>
       <c r="B112" s="16" t="s">
-        <v>382</v>
+        <v>388</v>
       </c>
       <c r="C112" s="17" t="s">
-        <v>432</v>
+        <v>438</v>
       </c>
       <c r="D112" s="17" t="s">
-        <v>433</v>
+        <v>439</v>
       </c>
       <c r="E112" s="17" t="s">
-        <v>434</v>
+        <v>440</v>
       </c>
       <c r="F112" s="18"/>
       <c r="G112" s="18"/>
@@ -5145,26 +5444,26 @@
     </row>
     <row r="113" s="1" customFormat="1" ht="15.75" customHeight="1" spans="1:9">
       <c r="A113" s="14" t="s">
-        <v>435</v>
+        <v>441</v>
       </c>
       <c r="H113" s="15"/>
       <c r="I113" s="15"/>
     </row>
     <row r="114" s="1" customFormat="1" ht="78.75" customHeight="1" spans="1:9">
       <c r="A114" s="16" t="s">
-        <v>436</v>
+        <v>442</v>
       </c>
       <c r="B114" s="16" t="s">
-        <v>393</v>
+        <v>399</v>
       </c>
       <c r="C114" s="17" t="s">
-        <v>437</v>
+        <v>443</v>
       </c>
       <c r="D114" s="17" t="s">
-        <v>438</v>
+        <v>444</v>
       </c>
       <c r="E114" s="17" t="s">
-        <v>439</v>
+        <v>445</v>
       </c>
       <c r="F114" s="18"/>
       <c r="G114" s="18"/>
@@ -5173,26 +5472,26 @@
     </row>
     <row r="115" s="1" customFormat="1" ht="15.75" customHeight="1" spans="1:9">
       <c r="A115" s="14" t="s">
-        <v>440</v>
+        <v>446</v>
       </c>
       <c r="H115" s="15"/>
       <c r="I115" s="15"/>
     </row>
     <row r="116" s="1" customFormat="1" ht="173.25" customHeight="1" spans="1:9">
       <c r="A116" s="16" t="s">
-        <v>441</v>
+        <v>447</v>
       </c>
       <c r="B116" s="16" t="s">
-        <v>442</v>
+        <v>448</v>
       </c>
       <c r="C116" s="17" t="s">
-        <v>443</v>
+        <v>449</v>
       </c>
       <c r="D116" s="17" t="s">
-        <v>444</v>
+        <v>450</v>
       </c>
       <c r="E116" s="17" t="s">
-        <v>445</v>
+        <v>451</v>
       </c>
       <c r="F116" s="18"/>
       <c r="G116" s="18"/>
@@ -5201,19 +5500,19 @@
     </row>
     <row r="117" s="1" customFormat="1" ht="141.75" customHeight="1" spans="1:9">
       <c r="A117" s="16" t="s">
-        <v>446</v>
+        <v>452</v>
       </c>
       <c r="B117" s="16" t="s">
-        <v>447</v>
+        <v>453</v>
       </c>
       <c r="C117" s="17" t="s">
-        <v>448</v>
+        <v>454</v>
       </c>
       <c r="D117" s="17" t="s">
-        <v>449</v>
+        <v>455</v>
       </c>
       <c r="E117" s="17" t="s">
-        <v>450</v>
+        <v>456</v>
       </c>
       <c r="F117" s="18"/>
       <c r="G117" s="18"/>
@@ -5222,19 +5521,19 @@
     </row>
     <row r="118" s="1" customFormat="1" ht="157.5" customHeight="1" spans="1:9">
       <c r="A118" s="16" t="s">
-        <v>451</v>
+        <v>457</v>
       </c>
       <c r="B118" s="16" t="s">
-        <v>452</v>
+        <v>458</v>
       </c>
       <c r="C118" s="17" t="s">
-        <v>453</v>
+        <v>459</v>
       </c>
       <c r="D118" s="17" t="s">
-        <v>454</v>
+        <v>460</v>
       </c>
       <c r="E118" s="17" t="s">
-        <v>455</v>
+        <v>461</v>
       </c>
       <c r="F118" s="18"/>
       <c r="G118" s="18"/>
@@ -5243,19 +5542,19 @@
     </row>
     <row r="119" s="1" customFormat="1" ht="141.75" customHeight="1" spans="1:9">
       <c r="A119" s="16" t="s">
-        <v>456</v>
+        <v>462</v>
       </c>
       <c r="B119" s="16" t="s">
-        <v>457</v>
+        <v>463</v>
       </c>
       <c r="C119" s="17" t="s">
-        <v>458</v>
+        <v>464</v>
       </c>
       <c r="D119" s="17" t="s">
-        <v>459</v>
+        <v>465</v>
       </c>
       <c r="E119" s="17" t="s">
-        <v>460</v>
+        <v>466</v>
       </c>
       <c r="F119" s="18"/>
       <c r="G119" s="18"/>
@@ -5264,19 +5563,19 @@
     </row>
     <row r="120" s="1" customFormat="1" ht="141.75" customHeight="1" spans="1:9">
       <c r="A120" s="16" t="s">
-        <v>461</v>
+        <v>467</v>
       </c>
       <c r="B120" s="16" t="s">
-        <v>125</v>
+        <v>128</v>
       </c>
       <c r="C120" s="17" t="s">
-        <v>462</v>
+        <v>468</v>
       </c>
       <c r="D120" s="17" t="s">
-        <v>463</v>
+        <v>469</v>
       </c>
       <c r="E120" s="17" t="s">
-        <v>464</v>
+        <v>470</v>
       </c>
       <c r="F120" s="18"/>
       <c r="G120" s="18"/>
@@ -5285,19 +5584,19 @@
     </row>
     <row r="121" s="1" customFormat="1" ht="78.75" customHeight="1" spans="1:9">
       <c r="A121" s="16" t="s">
-        <v>465</v>
+        <v>471</v>
       </c>
       <c r="B121" s="16" t="s">
-        <v>466</v>
+        <v>472</v>
       </c>
       <c r="C121" s="17" t="s">
-        <v>467</v>
+        <v>473</v>
       </c>
       <c r="D121" s="17" t="s">
-        <v>468</v>
+        <v>474</v>
       </c>
       <c r="E121" s="17" t="s">
-        <v>469</v>
+        <v>475</v>
       </c>
       <c r="F121" s="18"/>
       <c r="G121" s="18"/>
@@ -5306,26 +5605,26 @@
     </row>
     <row r="122" s="1" customFormat="1" ht="15.75" customHeight="1" spans="1:9">
       <c r="A122" s="14" t="s">
-        <v>470</v>
+        <v>476</v>
       </c>
       <c r="H122" s="15"/>
       <c r="I122" s="15"/>
     </row>
     <row r="123" s="1" customFormat="1" ht="78.75" customHeight="1" spans="1:9">
       <c r="A123" s="16" t="s">
-        <v>471</v>
+        <v>477</v>
       </c>
       <c r="B123" s="16" t="s">
-        <v>472</v>
+        <v>478</v>
       </c>
       <c r="C123" s="17" t="s">
-        <v>473</v>
+        <v>479</v>
       </c>
       <c r="D123" s="17" t="s">
-        <v>474</v>
+        <v>480</v>
       </c>
       <c r="E123" s="17" t="s">
-        <v>475</v>
+        <v>481</v>
       </c>
       <c r="F123" s="18"/>
       <c r="G123" s="18"/>
@@ -5334,19 +5633,19 @@
     </row>
     <row r="124" s="1" customFormat="1" ht="78.75" customHeight="1" spans="1:9">
       <c r="A124" s="16" t="s">
-        <v>476</v>
+        <v>482</v>
       </c>
       <c r="B124" s="16" t="s">
-        <v>466</v>
+        <v>472</v>
       </c>
       <c r="C124" s="17" t="s">
-        <v>477</v>
+        <v>483</v>
       </c>
       <c r="D124" s="17" t="s">
-        <v>478</v>
+        <v>484</v>
       </c>
       <c r="E124" s="17" t="s">
-        <v>479</v>
+        <v>485</v>
       </c>
       <c r="F124" s="18"/>
       <c r="G124" s="18"/>
@@ -5355,19 +5654,19 @@
     </row>
     <row r="125" s="1" customFormat="1" ht="78.75" customHeight="1" spans="1:9">
       <c r="A125" s="16" t="s">
-        <v>480</v>
+        <v>486</v>
       </c>
       <c r="B125" s="16" t="s">
-        <v>481</v>
+        <v>487</v>
       </c>
       <c r="C125" s="17" t="s">
-        <v>482</v>
+        <v>488</v>
       </c>
       <c r="D125" s="17" t="s">
-        <v>483</v>
+        <v>489</v>
       </c>
       <c r="E125" s="17" t="s">
-        <v>484</v>
+        <v>490</v>
       </c>
       <c r="F125" s="18"/>
       <c r="G125" s="18"/>
@@ -5376,19 +5675,19 @@
     </row>
     <row r="126" s="1" customFormat="1" ht="78.75" customHeight="1" spans="1:9">
       <c r="A126" s="16" t="s">
-        <v>485</v>
+        <v>491</v>
       </c>
       <c r="B126" s="16" t="s">
-        <v>377</v>
+        <v>383</v>
       </c>
       <c r="C126" s="17" t="s">
-        <v>486</v>
+        <v>492</v>
       </c>
       <c r="D126" s="17" t="s">
-        <v>487</v>
+        <v>493</v>
       </c>
       <c r="E126" s="17" t="s">
-        <v>488</v>
+        <v>494</v>
       </c>
       <c r="F126" s="18"/>
       <c r="G126" s="18"/>
@@ -5397,26 +5696,26 @@
     </row>
     <row r="127" s="1" customFormat="1" ht="15.75" customHeight="1" spans="1:9">
       <c r="A127" s="14" t="s">
-        <v>489</v>
+        <v>495</v>
       </c>
       <c r="H127" s="15"/>
       <c r="I127" s="15"/>
     </row>
     <row r="128" s="1" customFormat="1" ht="78.75" customHeight="1" spans="1:9">
       <c r="A128" s="16" t="s">
-        <v>490</v>
+        <v>496</v>
       </c>
       <c r="B128" s="16" t="s">
-        <v>491</v>
+        <v>497</v>
       </c>
       <c r="C128" s="17" t="s">
-        <v>492</v>
+        <v>498</v>
       </c>
       <c r="D128" s="17" t="s">
-        <v>493</v>
+        <v>499</v>
       </c>
       <c r="E128" s="17" t="s">
-        <v>494</v>
+        <v>500</v>
       </c>
       <c r="F128" s="18"/>
       <c r="G128" s="18"/>
@@ -5425,19 +5724,19 @@
     </row>
     <row r="129" s="1" customFormat="1" ht="78.75" customHeight="1" spans="1:9">
       <c r="A129" s="16" t="s">
-        <v>495</v>
+        <v>501</v>
       </c>
       <c r="B129" s="16" t="s">
-        <v>377</v>
+        <v>383</v>
       </c>
       <c r="C129" s="17" t="s">
-        <v>496</v>
+        <v>502</v>
       </c>
       <c r="D129" s="17" t="s">
-        <v>497</v>
+        <v>503</v>
       </c>
       <c r="E129" s="17" t="s">
-        <v>498</v>
+        <v>504</v>
       </c>
       <c r="F129" s="18"/>
       <c r="G129" s="18"/>
@@ -5446,19 +5745,19 @@
     </row>
     <row r="130" s="1" customFormat="1" ht="78.75" customHeight="1" spans="1:9">
       <c r="A130" s="16" t="s">
-        <v>499</v>
+        <v>505</v>
       </c>
       <c r="B130" s="16" t="s">
-        <v>500</v>
+        <v>506</v>
       </c>
       <c r="C130" s="17" t="s">
-        <v>501</v>
+        <v>507</v>
       </c>
       <c r="D130" s="17" t="s">
-        <v>502</v>
+        <v>508</v>
       </c>
       <c r="E130" s="17" t="s">
-        <v>503</v>
+        <v>509</v>
       </c>
       <c r="F130" s="18"/>
       <c r="G130" s="18"/>
@@ -5467,26 +5766,26 @@
     </row>
     <row r="131" s="1" customFormat="1" ht="15.75" customHeight="1" spans="1:9">
       <c r="A131" s="14" t="s">
-        <v>504</v>
+        <v>510</v>
       </c>
       <c r="H131" s="15"/>
       <c r="I131" s="15"/>
     </row>
     <row r="132" s="1" customFormat="1" ht="157.5" customHeight="1" spans="1:9">
       <c r="A132" s="17" t="s">
-        <v>505</v>
+        <v>511</v>
       </c>
       <c r="B132" s="17" t="s">
-        <v>506</v>
+        <v>512</v>
       </c>
       <c r="C132" s="17" t="s">
-        <v>507</v>
+        <v>513</v>
       </c>
       <c r="D132" s="17" t="s">
-        <v>508</v>
+        <v>514</v>
       </c>
       <c r="E132" s="17" t="s">
-        <v>509</v>
+        <v>515</v>
       </c>
       <c r="F132" s="18"/>
       <c r="G132" s="18"/>
@@ -5495,19 +5794,19 @@
     </row>
     <row r="133" s="1" customFormat="1" ht="220.5" customHeight="1" spans="1:9">
       <c r="A133" s="16" t="s">
-        <v>510</v>
+        <v>516</v>
       </c>
       <c r="B133" s="16" t="s">
-        <v>511</v>
+        <v>517</v>
       </c>
       <c r="C133" s="17" t="s">
-        <v>512</v>
+        <v>518</v>
       </c>
       <c r="D133" s="17" t="s">
-        <v>513</v>
+        <v>519</v>
       </c>
       <c r="E133" s="17" t="s">
-        <v>514</v>
+        <v>520</v>
       </c>
       <c r="F133" s="18"/>
       <c r="G133" s="18"/>
@@ -5516,19 +5815,19 @@
     </row>
     <row r="134" s="1" customFormat="1" ht="94.5" customHeight="1" spans="1:9">
       <c r="A134" s="17" t="s">
-        <v>515</v>
+        <v>521</v>
       </c>
       <c r="B134" s="17" t="s">
-        <v>516</v>
+        <v>522</v>
       </c>
       <c r="C134" s="17" t="s">
-        <v>517</v>
+        <v>523</v>
       </c>
       <c r="D134" s="17" t="s">
-        <v>518</v>
+        <v>524</v>
       </c>
       <c r="E134" s="17" t="s">
-        <v>519</v>
+        <v>525</v>
       </c>
       <c r="F134" s="18"/>
       <c r="G134" s="18"/>
@@ -5537,19 +5836,19 @@
     </row>
     <row r="135" s="1" customFormat="1" ht="141.75" customHeight="1" spans="1:9">
       <c r="A135" s="17" t="s">
-        <v>520</v>
+        <v>526</v>
       </c>
       <c r="B135" s="17" t="s">
-        <v>516</v>
+        <v>522</v>
       </c>
       <c r="C135" s="17" t="s">
-        <v>521</v>
+        <v>527</v>
       </c>
       <c r="D135" s="17" t="s">
-        <v>522</v>
+        <v>528</v>
       </c>
       <c r="E135" s="17" t="s">
-        <v>523</v>
+        <v>529</v>
       </c>
       <c r="F135" s="18"/>
       <c r="G135" s="18"/>
@@ -5558,19 +5857,19 @@
     </row>
     <row r="136" s="1" customFormat="1" ht="78.75" customHeight="1" spans="1:9">
       <c r="A136" s="16" t="s">
-        <v>524</v>
+        <v>530</v>
       </c>
       <c r="B136" s="16" t="s">
-        <v>525</v>
+        <v>531</v>
       </c>
       <c r="C136" s="17" t="s">
-        <v>526</v>
+        <v>532</v>
       </c>
       <c r="D136" s="17" t="s">
-        <v>527</v>
+        <v>533</v>
       </c>
       <c r="E136" s="17" t="s">
-        <v>528</v>
+        <v>534</v>
       </c>
       <c r="F136" s="18"/>
       <c r="G136" s="18"/>
@@ -5579,26 +5878,26 @@
     </row>
     <row r="137" s="1" customFormat="1" ht="15.75" customHeight="1" spans="1:9">
       <c r="A137" s="14" t="s">
-        <v>529</v>
+        <v>535</v>
       </c>
       <c r="H137" s="15"/>
       <c r="I137" s="15"/>
     </row>
     <row r="138" s="1" customFormat="1" ht="94.5" customHeight="1" spans="1:9">
       <c r="A138" s="16" t="s">
-        <v>530</v>
+        <v>536</v>
       </c>
       <c r="B138" s="16" t="s">
-        <v>531</v>
+        <v>537</v>
       </c>
       <c r="C138" s="17" t="s">
-        <v>532</v>
-      </c>
-      <c r="D138" s="17" t="s">
-        <v>533</v>
+        <v>538</v>
+      </c>
+      <c r="D138" s="20" t="s">
+        <v>539</v>
       </c>
       <c r="E138" s="17" t="s">
-        <v>534</v>
+        <v>540</v>
       </c>
       <c r="F138" s="18"/>
       <c r="G138" s="18"/>
@@ -5607,19 +5906,19 @@
     </row>
     <row r="139" s="1" customFormat="1" ht="94.5" customHeight="1" spans="1:9">
       <c r="A139" s="16" t="s">
-        <v>535</v>
+        <v>541</v>
       </c>
       <c r="B139" s="16" t="s">
-        <v>536</v>
+        <v>542</v>
       </c>
       <c r="C139" s="17" t="s">
-        <v>537</v>
-      </c>
-      <c r="D139" s="17" t="s">
-        <v>538</v>
+        <v>543</v>
+      </c>
+      <c r="D139" s="20" t="s">
+        <v>544</v>
       </c>
       <c r="E139" s="17" t="s">
-        <v>539</v>
+        <v>545</v>
       </c>
       <c r="F139" s="18"/>
       <c r="G139" s="18"/>
@@ -5628,19 +5927,19 @@
     </row>
     <row r="140" s="1" customFormat="1" ht="157.5" customHeight="1" spans="1:9">
       <c r="A140" s="16" t="s">
-        <v>540</v>
+        <v>546</v>
       </c>
       <c r="B140" s="16" t="s">
-        <v>531</v>
+        <v>537</v>
       </c>
       <c r="C140" s="17" t="s">
-        <v>541</v>
-      </c>
-      <c r="D140" s="17" t="s">
-        <v>542</v>
+        <v>547</v>
+      </c>
+      <c r="D140" s="20" t="s">
+        <v>548</v>
       </c>
       <c r="E140" s="17" t="s">
-        <v>543</v>
+        <v>549</v>
       </c>
       <c r="F140" s="18"/>
       <c r="G140" s="18"/>
@@ -5649,19 +5948,19 @@
     </row>
     <row r="141" s="1" customFormat="1" ht="220.5" customHeight="1" spans="1:9">
       <c r="A141" s="16" t="s">
-        <v>544</v>
+        <v>550</v>
       </c>
       <c r="B141" s="16" t="s">
-        <v>531</v>
+        <v>537</v>
       </c>
       <c r="C141" s="17" t="s">
-        <v>545</v>
+        <v>551</v>
       </c>
       <c r="D141" s="17" t="s">
-        <v>546</v>
+        <v>552</v>
       </c>
       <c r="E141" s="17" t="s">
-        <v>547</v>
+        <v>553</v>
       </c>
       <c r="F141" s="18"/>
       <c r="G141" s="18"/>
@@ -5670,19 +5969,19 @@
     </row>
     <row r="142" s="1" customFormat="1" ht="141.75" customHeight="1" spans="1:9">
       <c r="A142" s="16" t="s">
-        <v>548</v>
+        <v>554</v>
       </c>
       <c r="B142" s="16" t="s">
-        <v>531</v>
+        <v>537</v>
       </c>
       <c r="C142" s="17" t="s">
-        <v>549</v>
-      </c>
-      <c r="D142" s="17" t="s">
-        <v>550</v>
+        <v>555</v>
+      </c>
+      <c r="D142" s="20" t="s">
+        <v>556</v>
       </c>
       <c r="E142" s="17" t="s">
-        <v>551</v>
+        <v>557</v>
       </c>
       <c r="F142" s="18"/>
       <c r="G142" s="18"/>
@@ -5691,19 +5990,19 @@
     </row>
     <row r="143" s="1" customFormat="1" ht="141.75" customHeight="1" spans="1:9">
       <c r="A143" s="16" t="s">
-        <v>552</v>
+        <v>558</v>
       </c>
       <c r="B143" s="16" t="s">
-        <v>531</v>
+        <v>537</v>
       </c>
       <c r="C143" s="17" t="s">
-        <v>553</v>
-      </c>
-      <c r="D143" s="17" t="s">
-        <v>554</v>
+        <v>559</v>
+      </c>
+      <c r="D143" s="20" t="s">
+        <v>560</v>
       </c>
       <c r="E143" s="17" t="s">
-        <v>555</v>
+        <v>561</v>
       </c>
       <c r="F143" s="18"/>
       <c r="G143" s="18"/>
@@ -5712,19 +6011,19 @@
     </row>
     <row r="144" s="1" customFormat="1" ht="204.75" customHeight="1" spans="1:9">
       <c r="A144" s="16" t="s">
-        <v>556</v>
+        <v>562</v>
       </c>
       <c r="B144" s="16" t="s">
-        <v>531</v>
+        <v>537</v>
       </c>
       <c r="C144" s="17" t="s">
-        <v>557</v>
-      </c>
-      <c r="D144" s="17" t="s">
-        <v>558</v>
+        <v>563</v>
+      </c>
+      <c r="D144" s="20" t="s">
+        <v>564</v>
       </c>
       <c r="E144" s="17" t="s">
-        <v>559</v>
+        <v>565</v>
       </c>
       <c r="F144" s="18"/>
       <c r="G144" s="18"/>
@@ -5733,26 +6032,26 @@
     </row>
     <row r="145" s="1" customFormat="1" ht="15.75" customHeight="1" spans="1:9">
       <c r="A145" s="14" t="s">
-        <v>560</v>
+        <v>566</v>
       </c>
       <c r="H145" s="15"/>
       <c r="I145" s="15"/>
     </row>
     <row r="146" s="1" customFormat="1" ht="78.75" customHeight="1" spans="1:9">
       <c r="A146" s="16" t="s">
-        <v>561</v>
+        <v>567</v>
       </c>
       <c r="B146" s="16" t="s">
-        <v>562</v>
+        <v>568</v>
       </c>
       <c r="C146" s="17" t="s">
-        <v>563</v>
+        <v>569</v>
       </c>
       <c r="D146" s="17" t="s">
-        <v>564</v>
+        <v>570</v>
       </c>
       <c r="E146" s="17" t="s">
-        <v>565</v>
+        <v>571</v>
       </c>
       <c r="F146" s="18"/>
       <c r="G146" s="18"/>
@@ -5761,19 +6060,19 @@
     </row>
     <row r="147" s="1" customFormat="1" ht="78.75" customHeight="1" spans="1:9">
       <c r="A147" s="16" t="s">
-        <v>566</v>
+        <v>572</v>
       </c>
       <c r="B147" s="16" t="s">
-        <v>567</v>
+        <v>573</v>
       </c>
       <c r="C147" s="17" t="s">
-        <v>568</v>
+        <v>574</v>
       </c>
       <c r="D147" s="17" t="s">
-        <v>569</v>
+        <v>575</v>
       </c>
       <c r="E147" s="17" t="s">
-        <v>570</v>
+        <v>576</v>
       </c>
       <c r="F147" s="18"/>
       <c r="G147" s="18"/>
@@ -5782,26 +6081,26 @@
     </row>
     <row r="148" s="1" customFormat="1" ht="15.75" customHeight="1" spans="1:9">
       <c r="A148" s="14" t="s">
-        <v>571</v>
+        <v>577</v>
       </c>
       <c r="H148" s="15"/>
       <c r="I148" s="15"/>
     </row>
     <row r="149" s="1" customFormat="1" ht="126" customHeight="1" spans="1:9">
       <c r="A149" s="16" t="s">
-        <v>572</v>
+        <v>578</v>
       </c>
       <c r="B149" s="16" t="s">
-        <v>308</v>
+        <v>314</v>
       </c>
       <c r="C149" s="17" t="s">
-        <v>573</v>
+        <v>579</v>
       </c>
       <c r="D149" s="17" t="s">
-        <v>574</v>
+        <v>580</v>
       </c>
       <c r="E149" s="17" t="s">
-        <v>575</v>
+        <v>581</v>
       </c>
       <c r="F149" s="18"/>
       <c r="G149" s="18"/>
@@ -5810,19 +6109,19 @@
     </row>
     <row r="150" s="1" customFormat="1" ht="157.5" customHeight="1" spans="1:9">
       <c r="A150" s="16" t="s">
-        <v>576</v>
+        <v>582</v>
       </c>
       <c r="B150" s="16" t="s">
-        <v>308</v>
+        <v>314</v>
       </c>
       <c r="C150" s="17" t="s">
-        <v>577</v>
+        <v>583</v>
       </c>
       <c r="D150" s="17" t="s">
-        <v>578</v>
+        <v>584</v>
       </c>
       <c r="E150" s="17" t="s">
-        <v>579</v>
+        <v>585</v>
       </c>
       <c r="F150" s="18"/>
       <c r="G150" s="18"/>
@@ -5831,19 +6130,19 @@
     </row>
     <row r="151" s="1" customFormat="1" ht="189" customHeight="1" spans="1:9">
       <c r="A151" s="16" t="s">
-        <v>580</v>
+        <v>586</v>
       </c>
       <c r="B151" s="16" t="s">
-        <v>581</v>
+        <v>587</v>
       </c>
       <c r="C151" s="17" t="s">
-        <v>582</v>
+        <v>588</v>
       </c>
       <c r="D151" s="17" t="s">
-        <v>583</v>
+        <v>589</v>
       </c>
       <c r="E151" s="17" t="s">
-        <v>584</v>
+        <v>590</v>
       </c>
       <c r="F151" s="18"/>
       <c r="G151" s="18"/>
@@ -5852,19 +6151,19 @@
     </row>
     <row r="152" s="1" customFormat="1" ht="157.5" customHeight="1" spans="1:9">
       <c r="A152" s="16" t="s">
-        <v>585</v>
+        <v>591</v>
       </c>
       <c r="B152" s="16" t="s">
-        <v>581</v>
+        <v>587</v>
       </c>
       <c r="C152" s="17" t="s">
-        <v>586</v>
+        <v>592</v>
       </c>
       <c r="D152" s="17" t="s">
-        <v>587</v>
+        <v>593</v>
       </c>
       <c r="E152" s="17" t="s">
-        <v>588</v>
+        <v>594</v>
       </c>
       <c r="F152" s="18"/>
       <c r="G152" s="18"/>
@@ -5873,19 +6172,19 @@
     </row>
     <row r="153" s="1" customFormat="1" ht="141.75" customHeight="1" spans="1:9">
       <c r="A153" s="16" t="s">
-        <v>589</v>
+        <v>595</v>
       </c>
       <c r="B153" s="16" t="s">
-        <v>590</v>
+        <v>596</v>
       </c>
       <c r="C153" s="17" t="s">
-        <v>591</v>
+        <v>597</v>
       </c>
       <c r="D153" s="17" t="s">
-        <v>592</v>
+        <v>598</v>
       </c>
       <c r="E153" s="17" t="s">
-        <v>593</v>
+        <v>599</v>
       </c>
       <c r="F153" s="18"/>
       <c r="G153" s="18"/>
@@ -5894,19 +6193,19 @@
     </row>
     <row r="154" ht="189" customHeight="1" spans="1:9">
       <c r="A154" s="16" t="s">
-        <v>594</v>
+        <v>600</v>
       </c>
       <c r="B154" s="16" t="s">
-        <v>595</v>
+        <v>601</v>
       </c>
       <c r="C154" s="17" t="s">
-        <v>596</v>
+        <v>602</v>
       </c>
       <c r="D154" s="17" t="s">
-        <v>597</v>
+        <v>603</v>
       </c>
       <c r="E154" s="17" t="s">
-        <v>598</v>
+        <v>604</v>
       </c>
       <c r="F154" s="18"/>
       <c r="G154" s="18"/>
@@ -5915,26 +6214,26 @@
     </row>
     <row r="155" ht="15.75" customHeight="1" spans="1:9">
       <c r="A155" s="14" t="s">
-        <v>599</v>
+        <v>605</v>
       </c>
       <c r="H155" s="15"/>
       <c r="I155" s="15"/>
     </row>
     <row r="156" ht="157.5" customHeight="1" spans="1:9">
       <c r="A156" s="16" t="s">
-        <v>600</v>
+        <v>606</v>
       </c>
       <c r="B156" s="16" t="s">
-        <v>531</v>
+        <v>537</v>
       </c>
       <c r="C156" s="17" t="s">
-        <v>249</v>
+        <v>254</v>
       </c>
       <c r="D156" s="17" t="s">
-        <v>250</v>
+        <v>255</v>
       </c>
       <c r="E156" s="17" t="s">
-        <v>601</v>
+        <v>607</v>
       </c>
       <c r="F156" s="18"/>
       <c r="G156" s="18"/>
@@ -5943,19 +6242,19 @@
     </row>
     <row r="157" ht="252" customHeight="1" spans="1:9">
       <c r="A157" s="16" t="s">
-        <v>602</v>
+        <v>608</v>
       </c>
       <c r="B157" s="16" t="s">
-        <v>603</v>
+        <v>609</v>
       </c>
       <c r="C157" s="17" t="s">
-        <v>604</v>
+        <v>610</v>
       </c>
       <c r="D157" s="17" t="s">
-        <v>605</v>
+        <v>611</v>
       </c>
       <c r="E157" s="17" t="s">
-        <v>606</v>
+        <v>612</v>
       </c>
       <c r="F157" s="18"/>
       <c r="G157" s="18"/>
@@ -5964,19 +6263,19 @@
     </row>
     <row r="158" ht="220.5" customHeight="1" spans="1:9">
       <c r="A158" s="16" t="s">
-        <v>607</v>
+        <v>613</v>
       </c>
       <c r="B158" s="16" t="s">
-        <v>603</v>
+        <v>609</v>
       </c>
       <c r="C158" s="17" t="s">
-        <v>608</v>
+        <v>614</v>
       </c>
       <c r="D158" s="17" t="s">
-        <v>609</v>
+        <v>615</v>
       </c>
       <c r="E158" s="17" t="s">
-        <v>610</v>
+        <v>616</v>
       </c>
       <c r="F158" s="18"/>
       <c r="G158" s="18"/>
@@ -5985,19 +6284,19 @@
     </row>
     <row r="159" ht="204.75" customHeight="1" spans="1:9">
       <c r="A159" s="17" t="s">
-        <v>611</v>
+        <v>617</v>
       </c>
       <c r="B159" s="17" t="s">
-        <v>101</v>
+        <v>104</v>
       </c>
       <c r="C159" s="17" t="s">
-        <v>612</v>
+        <v>618</v>
       </c>
       <c r="D159" s="17" t="s">
-        <v>233</v>
+        <v>238</v>
       </c>
       <c r="E159" s="17" t="s">
-        <v>613</v>
+        <v>619</v>
       </c>
       <c r="F159" s="18"/>
       <c r="G159" s="18"/>
@@ -6006,19 +6305,19 @@
     </row>
     <row r="160" ht="126" customHeight="1" spans="1:9">
       <c r="A160" s="16" t="s">
-        <v>614</v>
+        <v>620</v>
       </c>
       <c r="B160" s="16" t="s">
-        <v>531</v>
+        <v>537</v>
       </c>
       <c r="C160" s="17" t="s">
-        <v>615</v>
+        <v>621</v>
       </c>
       <c r="D160" s="17" t="s">
-        <v>616</v>
+        <v>622</v>
       </c>
       <c r="E160" s="17" t="s">
-        <v>617</v>
+        <v>623</v>
       </c>
       <c r="F160" s="18"/>
       <c r="G160" s="18"/>
@@ -6027,19 +6326,19 @@
     </row>
     <row r="161" ht="78.75" customHeight="1" spans="1:9">
       <c r="A161" s="16" t="s">
-        <v>618</v>
+        <v>624</v>
       </c>
       <c r="B161" s="16" t="s">
-        <v>393</v>
+        <v>399</v>
       </c>
       <c r="C161" s="17" t="s">
-        <v>619</v>
+        <v>625</v>
       </c>
       <c r="D161" s="17" t="s">
-        <v>620</v>
+        <v>626</v>
       </c>
       <c r="E161" s="17" t="s">
-        <v>621</v>
+        <v>627</v>
       </c>
       <c r="F161" s="18"/>
       <c r="G161" s="18"/>
@@ -6048,26 +6347,26 @@
     </row>
     <row r="162" ht="15.75" customHeight="1" spans="1:9">
       <c r="A162" s="14" t="s">
-        <v>622</v>
+        <v>628</v>
       </c>
       <c r="H162" s="15"/>
       <c r="I162" s="15"/>
     </row>
     <row r="163" ht="157.5" customHeight="1" spans="1:9">
       <c r="A163" s="16" t="s">
-        <v>623</v>
+        <v>629</v>
       </c>
       <c r="B163" s="16" t="s">
-        <v>624</v>
+        <v>630</v>
       </c>
       <c r="C163" s="17" t="s">
-        <v>625</v>
+        <v>631</v>
       </c>
       <c r="D163" s="17" t="s">
-        <v>626</v>
+        <v>632</v>
       </c>
       <c r="E163" s="17" t="s">
-        <v>627</v>
+        <v>633</v>
       </c>
       <c r="F163" s="18"/>
       <c r="G163" s="18"/>
@@ -6110,15 +6409,45 @@
     <mergeCell ref="A162:G162"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink ref="C6" r:id="rId1" display="Avinox stellt neuen MG Concept Motor vor"/>
-    <hyperlink ref="C7" r:id="rId2" display="Avinox MG Concept: Lightweight, Full-Power Combined eBike Motor &amp; Gearbox Project"/>
-    <hyperlink ref="D8" r:id="rId3" display="https://ebike-mtb.com/en/avinox-mg-gearbox-motor/"/>
-    <hyperlink ref="D9" r:id="rId4" display="https://www.avinox-ebike.com/drive-unit?from=nav&amp;site=avinox-ebike"/>
-    <hyperlink ref="D10" r:id="rId5" display="https://www.avinox-ebike.com/news/avinox-concept-product-eurobike-2026"/>
+    <hyperlink ref="C6" r:id="rId2" display="Avinox stellt neuen MG Concept Motor vor"/>
+    <hyperlink ref="C7" r:id="rId3" display="Avinox MG Concept: Lightweight, Full-Power Combined eBike Motor &amp; Gearbox Project"/>
+    <hyperlink ref="D8" r:id="rId4" display="https://ebike-mtb.com/en/avinox-mg-gearbox-motor/"/>
+    <hyperlink ref="D9" r:id="rId5" display="https://www.avinox-ebike.com/drive-unit?from=nav&amp;site=avinox-ebike"/>
+    <hyperlink ref="D10" r:id="rId6" display="https://www.avinox-ebike.com/news/avinox-concept-product-eurobike-2026"/>
+    <hyperlink ref="D13" r:id="rId7" display="https://gobao-ebike.com/x-system-new/"/>
+    <hyperlink ref="D14" r:id="rId8" display="https://www.theverge.com/news/959382/avinox-mg-concept-gobao-mgu-ecvt"/>
+    <hyperlink ref="D15" r:id="rId9" display="https://www.transitionvelo.com/composants/moteurs-batteries/moteurs/gobao-x1-et-x1p-ecvt-les-nouveaux-monstres-chinois-qui-veulent-deja-detroner-avinox-et-owuru/"/>
+    <hyperlink ref="D16" r:id="rId10" display="https://bikebiz.com/gobao-introduces-the-x-e-bike-system-featuring-an-integrated-motor/"/>
+    <hyperlink ref="D17" r:id="rId11" display="https://ebike-mtb.com/en/gobao-x1p-review/"/>
+    <hyperlink ref="D19" r:id="rId12" display="https://pinion.eu/en/e-drive/"/>
+    <hyperlink ref="D20" r:id="rId13" display="https://pinion.eu/en/e-drive/smartshift-functions/"/>
+    <hyperlink ref="D22" r:id="rId14" display="https://pinion.eu/en/e-bikes/e-trekking/"/>
+    <hyperlink ref="D23" r:id="rId15" display="https://www.simplon.com/en/Bikes/Trekking-Bikes/KAGU-ePinion-High_b_915075"/>
+    <hyperlink ref="D24" r:id="rId16" display="https://www.simplon.com/en/Bikes/E-Mountain-Bikes/Rapcon-ePinion_b_929057"/>
+    <hyperlink ref="D25" r:id="rId17" display="https://www.welt.de/motor/news/article68ee16199bc2a314d86ea8dd/test-simplon-kagu-epinion-high.html"/>
+    <hyperlink ref="D26" r:id="rId18" display="https://www.radfahren.de/test-technik/simplon-kagu-epinion-high-test/"/>
+    <hyperlink ref="D27" r:id="rId19" display="https://www.welt.de/motor/news/article254225108/Flyer-Upstreet-TR-CF-7-63-Erstes-Fahrzeug-mit-neuem-Pinion-E-Bike-Antrieb.html"/>
+    <hyperlink ref="D29" r:id="rId20" display="https://pinion.eu/en/gearboxes/"/>
+    <hyperlink ref="D30" r:id="rId21" display="https://pinion.eu/en/p-line/"/>
+    <hyperlink ref="D32" r:id="rId22" display="https://www.bosch-ebike.com/en/products/eshift"/>
+    <hyperlink ref="D33" r:id="rId23" display="https://ebike-mtb.com/en/bosch-eshift-review-2024/"/>
+    <hyperlink ref="D46" r:id="rId24" display="https://www.theverge.com/23775103/veloretti-ace-two-ebike-review-price-specs"/>
+    <hyperlink ref="D77" r:id="rId25" display="https://www.pinkbike.com/news/why-ecvts-could-be-the-future-of-e-bike-drivetrains.html"/>
+    <hyperlink ref="D102" r:id="rId26" display="https://www.youtube.com/watch?v=0i5AsEzsP6Y"/>
+    <hyperlink ref="D103" r:id="rId27" display="https://www.youtube.com/watch?v=QENBAjQKUto"/>
+    <hyperlink ref="D138" r:id="rId28" display="https://enduro-mtb.com/en/classified-powershift-review/"/>
+    <hyperlink ref="D139" r:id="rId29" display="https://www.classified-cycling.cc/pages/white-papers"/>
+    <hyperlink ref="D140" r:id="rId30" display="https://www.cyclingweekly.com/reviews/the-classified-powershift-system-a-gravel-review"/>
+    <hyperlink ref="D142" r:id="rId31" display="https://www.ambmag.com.au/feature/classified-powershift-mtb-review-who-is-this-for/"/>
+    <hyperlink ref="D143" r:id="rId32" display="https://www.mbr.co.uk/reviews/wheelsets/classified-powershift-hub-gear-review"/>
+    <hyperlink ref="D144" r:id="rId33" display="https://www.bike-magazin.de/en/components/gearsticks/classified-powershift-the-new-two-speed-hub-for-mtb-in-the-test/"/>
+    <hyperlink ref="D89" r:id="rId11" display="https://ebike-mtb.com/en/gobao-x1p-review/"/>
+    <hyperlink ref="D79" r:id="rId4" display="https://ebike-mtb.com/en/avinox-mg-gearbox-motor/"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait"/>
   <headerFooter/>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
Add e-CVT rider feel visualization materials
</commit_message>
<xml_diff>
--- a/research-mgu/03_analysis/网页重点内容提取_后续与AI对比.xlsx
+++ b/research-mgu/03_analysis/网页重点内容提取_后续与AI对比.xlsx
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="774" uniqueCount="634">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="778" uniqueCount="636">
   <si>
     <t>SourceID</t>
   </si>
@@ -1125,6 +1125,9 @@
     <t>已写入正文；E-MOUNTAINBIKE 可补试骑/功能叙事</t>
   </si>
   <si>
+    <t>无论你是在攀爬陡坡、沿着流畅的小径巡航，还是快速换乘区段，你偏好的预设节奏都应保持基本不变。据Avinox介绍，这带来了极为平顺自然的骑行体验，因为辅助水平和传动比都会根据具体情况不断调整。</t>
+  </si>
+  <si>
     <t>6.1-002</t>
   </si>
   <si>
@@ -1240,6 +1243,9 @@
   </si>
   <si>
     <t>已写入正文；补 Eurobike 2026 与 X1P 试骑/评价语境</t>
+  </si>
+  <si>
+    <t>最引人注目的是即时且清晰的动力传输。即使在低踏频下，扭矩依然充足，加速极快且可控，最高可达25公里/小时的辅助限制。由于没有换挡，动力输出始终稳定且异常平稳。起始也非常简单且明确。</t>
   </si>
   <si>
     <t>6.2-002</t>
@@ -4786,26 +4792,32 @@
       <c r="E79" s="16" t="s">
         <v>312</v>
       </c>
-      <c r="F79" s="18"/>
+      <c r="F79" s="18" t="s">
+        <v>313</v>
+      </c>
       <c r="G79" s="18"/>
-      <c r="H79" s="15"/>
-      <c r="I79" s="15"/>
+      <c r="H79" s="15" t="s">
+        <v>17</v>
+      </c>
+      <c r="I79" s="15" t="s">
+        <v>17</v>
+      </c>
     </row>
     <row r="80" s="1" customFormat="1" ht="173.25" customHeight="1" spans="1:9">
       <c r="A80" s="16" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="B80" s="16" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="C80" s="17" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="D80" s="17" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="E80" s="17" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="F80" s="18"/>
       <c r="G80" s="18"/>
@@ -4814,19 +4826,19 @@
     </row>
     <row r="81" s="1" customFormat="1" ht="157.5" customHeight="1" spans="1:9">
       <c r="A81" s="16" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="B81" s="16" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="C81" s="17" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
       <c r="D81" s="17" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="E81" s="17" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="F81" s="18"/>
       <c r="G81" s="18"/>
@@ -4835,19 +4847,19 @@
     </row>
     <row r="82" s="1" customFormat="1" ht="220.5" customHeight="1" spans="1:9">
       <c r="A82" s="16" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="B82" s="16" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="C82" s="17" t="s">
-        <v>323</v>
+        <v>324</v>
       </c>
       <c r="D82" s="17" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="E82" s="17" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="F82" s="18"/>
       <c r="G82" s="18"/>
@@ -4856,10 +4868,10 @@
     </row>
     <row r="83" s="1" customFormat="1" ht="126" customHeight="1" spans="1:9">
       <c r="A83" s="16" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="B83" s="16" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="C83" s="17" t="s">
         <v>50</v>
@@ -4868,7 +4880,7 @@
         <v>51</v>
       </c>
       <c r="E83" s="17" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="F83" s="18"/>
       <c r="G83" s="18"/>
@@ -4877,19 +4889,19 @@
     </row>
     <row r="84" s="1" customFormat="1" ht="78.75" customHeight="1" spans="1:9">
       <c r="A84" s="16" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="B84" s="16" t="s">
-        <v>330</v>
+        <v>331</v>
       </c>
       <c r="C84" s="17" t="s">
-        <v>331</v>
+        <v>332</v>
       </c>
       <c r="D84" s="17" t="s">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="E84" s="17" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="F84" s="18"/>
       <c r="G84" s="18"/>
@@ -4898,19 +4910,19 @@
     </row>
     <row r="85" s="1" customFormat="1" ht="78.75" customHeight="1" spans="1:9">
       <c r="A85" s="16" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="B85" s="16" t="s">
-        <v>330</v>
+        <v>331</v>
       </c>
       <c r="C85" s="17" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="D85" s="17" t="s">
-        <v>336</v>
+        <v>337</v>
       </c>
       <c r="E85" s="17" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="F85" s="18"/>
       <c r="G85" s="18"/>
@@ -4919,19 +4931,19 @@
     </row>
     <row r="86" s="1" customFormat="1" ht="78.75" customHeight="1" spans="1:9">
       <c r="A86" s="16" t="s">
-        <v>338</v>
+        <v>339</v>
       </c>
       <c r="B86" s="16" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="C86" s="17" t="s">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="D86" s="17" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="E86" s="17" t="s">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="F86" s="18"/>
       <c r="G86" s="18"/>
@@ -4940,19 +4952,19 @@
     </row>
     <row r="87" s="1" customFormat="1" ht="78.75" customHeight="1" spans="1:9">
       <c r="A87" s="16" t="s">
-        <v>343</v>
+        <v>344</v>
       </c>
       <c r="B87" s="16" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="C87" s="17" t="s">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="D87" s="17" t="s">
-        <v>345</v>
+        <v>346</v>
       </c>
       <c r="E87" s="17" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="F87" s="18"/>
       <c r="G87" s="18"/>
@@ -4961,47 +4973,49 @@
     </row>
     <row r="88" s="1" customFormat="1" ht="15.75" customHeight="1" spans="1:9">
       <c r="A88" s="14" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="H88" s="15"/>
       <c r="I88" s="15"/>
     </row>
     <row r="89" s="1" customFormat="1" ht="78.75" customHeight="1" spans="1:9">
       <c r="A89" s="16" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="B89" s="16" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="C89" s="17" t="s">
-        <v>350</v>
-      </c>
-      <c r="D89" s="20" t="s">
+        <v>351</v>
+      </c>
+      <c r="D89" s="21" t="s">
         <v>79</v>
       </c>
       <c r="E89" s="16" t="s">
-        <v>351</v>
-      </c>
-      <c r="F89" s="18"/>
+        <v>352</v>
+      </c>
+      <c r="F89" s="18" t="s">
+        <v>353</v>
+      </c>
       <c r="G89" s="18"/>
       <c r="H89" s="15"/>
       <c r="I89" s="15"/>
     </row>
     <row r="90" s="1" customFormat="1" ht="173.25" customHeight="1" spans="1:9">
       <c r="A90" s="16" t="s">
-        <v>352</v>
+        <v>354</v>
       </c>
       <c r="B90" s="16" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="C90" s="17" t="s">
-        <v>353</v>
+        <v>355</v>
       </c>
       <c r="D90" s="17" t="s">
-        <v>354</v>
+        <v>356</v>
       </c>
       <c r="E90" s="17" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="F90" s="18"/>
       <c r="G90" s="18"/>
@@ -5010,19 +5024,19 @@
     </row>
     <row r="91" s="1" customFormat="1" ht="94.5" customHeight="1" spans="1:9">
       <c r="A91" s="16" t="s">
-        <v>355</v>
+        <v>357</v>
       </c>
       <c r="B91" s="16" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="C91" s="17" t="s">
-        <v>356</v>
+        <v>358</v>
       </c>
       <c r="D91" s="17" t="s">
-        <v>357</v>
+        <v>359</v>
       </c>
       <c r="E91" s="17" t="s">
-        <v>358</v>
+        <v>360</v>
       </c>
       <c r="F91" s="18"/>
       <c r="G91" s="18"/>
@@ -5031,19 +5045,19 @@
     </row>
     <row r="92" s="1" customFormat="1" ht="220.5" customHeight="1" spans="1:9">
       <c r="A92" s="16" t="s">
-        <v>359</v>
+        <v>361</v>
       </c>
       <c r="B92" s="16" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="C92" s="17" t="s">
-        <v>360</v>
+        <v>362</v>
       </c>
       <c r="D92" s="17" t="s">
-        <v>361</v>
+        <v>363</v>
       </c>
       <c r="E92" s="17" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="F92" s="18"/>
       <c r="G92" s="18"/>
@@ -5052,19 +5066,19 @@
     </row>
     <row r="93" s="1" customFormat="1" ht="141.75" customHeight="1" spans="1:9">
       <c r="A93" s="16" t="s">
-        <v>362</v>
+        <v>364</v>
       </c>
       <c r="B93" s="16" t="s">
-        <v>363</v>
+        <v>365</v>
       </c>
       <c r="C93" s="17" t="s">
-        <v>364</v>
+        <v>366</v>
       </c>
       <c r="D93" s="17" t="s">
-        <v>365</v>
+        <v>367</v>
       </c>
       <c r="E93" s="17" t="s">
-        <v>366</v>
+        <v>368</v>
       </c>
       <c r="F93" s="18"/>
       <c r="G93" s="18"/>
@@ -5073,19 +5087,19 @@
     </row>
     <row r="94" s="1" customFormat="1" ht="173.25" customHeight="1" spans="1:9">
       <c r="A94" s="16" t="s">
-        <v>367</v>
+        <v>369</v>
       </c>
       <c r="B94" s="16" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="C94" s="17" t="s">
-        <v>368</v>
+        <v>370</v>
       </c>
       <c r="D94" s="17" t="s">
-        <v>369</v>
+        <v>371</v>
       </c>
       <c r="E94" s="17" t="s">
-        <v>370</v>
+        <v>372</v>
       </c>
       <c r="F94" s="18"/>
       <c r="G94" s="18"/>
@@ -5094,19 +5108,19 @@
     </row>
     <row r="95" s="1" customFormat="1" ht="173.25" customHeight="1" spans="1:9">
       <c r="A95" s="16" t="s">
-        <v>371</v>
+        <v>373</v>
       </c>
       <c r="B95" s="16" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="C95" s="17" t="s">
-        <v>372</v>
+        <v>374</v>
       </c>
       <c r="D95" s="17" t="s">
-        <v>373</v>
+        <v>375</v>
       </c>
       <c r="E95" s="17" t="s">
-        <v>374</v>
+        <v>376</v>
       </c>
       <c r="F95" s="18"/>
       <c r="G95" s="18"/>
@@ -5115,19 +5129,19 @@
     </row>
     <row r="96" s="1" customFormat="1" ht="126" customHeight="1" spans="1:9">
       <c r="A96" s="16" t="s">
-        <v>375</v>
+        <v>377</v>
       </c>
       <c r="B96" s="16" t="s">
-        <v>363</v>
+        <v>365</v>
       </c>
       <c r="C96" s="17" t="s">
-        <v>376</v>
+        <v>378</v>
       </c>
       <c r="D96" s="17" t="s">
-        <v>377</v>
+        <v>379</v>
       </c>
       <c r="E96" s="17" t="s">
-        <v>378</v>
+        <v>380</v>
       </c>
       <c r="F96" s="18"/>
       <c r="G96" s="18"/>
@@ -5136,19 +5150,19 @@
     </row>
     <row r="97" s="1" customFormat="1" ht="78.75" customHeight="1" spans="1:9">
       <c r="A97" s="16" t="s">
-        <v>379</v>
+        <v>381</v>
       </c>
       <c r="B97" s="16" t="s">
-        <v>330</v>
+        <v>331</v>
       </c>
       <c r="C97" s="17" t="s">
-        <v>380</v>
+        <v>382</v>
       </c>
       <c r="D97" s="17" t="s">
-        <v>381</v>
+        <v>383</v>
       </c>
       <c r="E97" s="17" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="F97" s="18"/>
       <c r="G97" s="18"/>
@@ -5157,19 +5171,19 @@
     </row>
     <row r="98" s="1" customFormat="1" ht="78.75" customHeight="1" spans="1:9">
       <c r="A98" s="16" t="s">
-        <v>382</v>
+        <v>384</v>
       </c>
       <c r="B98" s="16" t="s">
-        <v>383</v>
+        <v>385</v>
       </c>
       <c r="C98" s="17" t="s">
-        <v>384</v>
+        <v>386</v>
       </c>
       <c r="D98" s="17" t="s">
-        <v>385</v>
+        <v>387</v>
       </c>
       <c r="E98" s="17" t="s">
-        <v>386</v>
+        <v>388</v>
       </c>
       <c r="F98" s="18"/>
       <c r="G98" s="18"/>
@@ -5178,19 +5192,19 @@
     </row>
     <row r="99" s="1" customFormat="1" ht="78.75" customHeight="1" spans="1:9">
       <c r="A99" s="16" t="s">
-        <v>387</v>
+        <v>389</v>
       </c>
       <c r="B99" s="16" t="s">
-        <v>388</v>
+        <v>390</v>
       </c>
       <c r="C99" s="17" t="s">
-        <v>389</v>
+        <v>391</v>
       </c>
       <c r="D99" s="17" t="s">
-        <v>390</v>
+        <v>392</v>
       </c>
       <c r="E99" s="17" t="s">
-        <v>391</v>
+        <v>393</v>
       </c>
       <c r="F99" s="18"/>
       <c r="G99" s="18"/>
@@ -5199,26 +5213,26 @@
     </row>
     <row r="100" s="1" customFormat="1" ht="15.75" customHeight="1" spans="1:9">
       <c r="A100" s="14" t="s">
-        <v>392</v>
+        <v>394</v>
       </c>
       <c r="H100" s="15"/>
       <c r="I100" s="15"/>
     </row>
     <row r="101" s="1" customFormat="1" ht="78.75" customHeight="1" spans="1:9">
       <c r="A101" s="16" t="s">
-        <v>393</v>
+        <v>395</v>
       </c>
       <c r="B101" s="16" t="s">
-        <v>394</v>
+        <v>396</v>
       </c>
       <c r="C101" s="17" t="s">
-        <v>395</v>
+        <v>397</v>
       </c>
       <c r="D101" s="17" t="s">
-        <v>396</v>
+        <v>398</v>
       </c>
       <c r="E101" s="17" t="s">
-        <v>397</v>
+        <v>399</v>
       </c>
       <c r="F101" s="18"/>
       <c r="G101" s="18"/>
@@ -5227,19 +5241,19 @@
     </row>
     <row r="102" s="1" customFormat="1" ht="78.75" customHeight="1" spans="1:9">
       <c r="A102" s="16" t="s">
-        <v>398</v>
+        <v>400</v>
       </c>
       <c r="B102" s="16" t="s">
-        <v>399</v>
+        <v>401</v>
       </c>
       <c r="C102" s="17" t="s">
-        <v>400</v>
-      </c>
-      <c r="D102" s="20" t="s">
-        <v>401</v>
+        <v>402</v>
+      </c>
+      <c r="D102" s="21" t="s">
+        <v>403</v>
       </c>
       <c r="E102" s="17" t="s">
-        <v>402</v>
+        <v>404</v>
       </c>
       <c r="F102" s="18"/>
       <c r="G102" s="18"/>
@@ -5248,19 +5262,19 @@
     </row>
     <row r="103" s="1" customFormat="1" ht="78.75" customHeight="1" spans="1:9">
       <c r="A103" s="16" t="s">
-        <v>403</v>
+        <v>405</v>
       </c>
       <c r="B103" s="16" t="s">
-        <v>394</v>
+        <v>396</v>
       </c>
       <c r="C103" s="17" t="s">
-        <v>404</v>
+        <v>406</v>
       </c>
       <c r="D103" s="20" t="s">
-        <v>405</v>
+        <v>407</v>
       </c>
       <c r="E103" s="17" t="s">
-        <v>406</v>
+        <v>408</v>
       </c>
       <c r="F103" s="18"/>
       <c r="G103" s="18"/>
@@ -5269,10 +5283,10 @@
     </row>
     <row r="104" s="1" customFormat="1" ht="78.75" customHeight="1" spans="1:9">
       <c r="A104" s="16" t="s">
-        <v>407</v>
+        <v>409</v>
       </c>
       <c r="B104" s="16" t="s">
-        <v>408</v>
+        <v>410</v>
       </c>
       <c r="C104" s="17" t="s">
         <v>246</v>
@@ -5281,7 +5295,7 @@
         <v>247</v>
       </c>
       <c r="E104" s="16" t="s">
-        <v>409</v>
+        <v>411</v>
       </c>
       <c r="F104" s="18"/>
       <c r="G104" s="18"/>
@@ -5290,17 +5304,17 @@
     </row>
     <row r="105" s="1" customFormat="1" ht="15.75" customHeight="1" spans="1:9">
       <c r="A105" s="14" t="s">
-        <v>410</v>
+        <v>412</v>
       </c>
       <c r="H105" s="15"/>
       <c r="I105" s="15"/>
     </row>
     <row r="106" s="1" customFormat="1" ht="94.5" customHeight="1" spans="1:9">
       <c r="A106" s="16" t="s">
-        <v>411</v>
+        <v>413</v>
       </c>
       <c r="B106" s="16" t="s">
-        <v>412</v>
+        <v>414</v>
       </c>
       <c r="C106" s="17" t="s">
         <v>145</v>
@@ -5309,7 +5323,7 @@
         <v>146</v>
       </c>
       <c r="E106" s="16" t="s">
-        <v>413</v>
+        <v>415</v>
       </c>
       <c r="F106" s="18"/>
       <c r="G106" s="18"/>
@@ -5318,19 +5332,19 @@
     </row>
     <row r="107" s="1" customFormat="1" ht="252" customHeight="1" spans="1:9">
       <c r="A107" s="16" t="s">
-        <v>414</v>
+        <v>416</v>
       </c>
       <c r="B107" s="16" t="s">
-        <v>415</v>
+        <v>417</v>
       </c>
       <c r="C107" s="17" t="s">
-        <v>416</v>
+        <v>418</v>
       </c>
       <c r="D107" s="17" t="s">
-        <v>417</v>
+        <v>419</v>
       </c>
       <c r="E107" s="17" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="F107" s="18"/>
       <c r="G107" s="18"/>
@@ -5339,19 +5353,19 @@
     </row>
     <row r="108" s="1" customFormat="1" ht="236.25" customHeight="1" spans="1:9">
       <c r="A108" s="16" t="s">
-        <v>418</v>
+        <v>420</v>
       </c>
       <c r="B108" s="16" t="s">
-        <v>419</v>
+        <v>421</v>
       </c>
       <c r="C108" s="17" t="s">
-        <v>420</v>
+        <v>422</v>
       </c>
       <c r="D108" s="17" t="s">
-        <v>421</v>
+        <v>423</v>
       </c>
       <c r="E108" s="17" t="s">
-        <v>422</v>
+        <v>424</v>
       </c>
       <c r="F108" s="18"/>
       <c r="G108" s="18"/>
@@ -5360,19 +5374,19 @@
     </row>
     <row r="109" s="1" customFormat="1" ht="141.75" customHeight="1" spans="1:9">
       <c r="A109" s="16" t="s">
-        <v>423</v>
+        <v>425</v>
       </c>
       <c r="B109" s="16" t="s">
-        <v>424</v>
+        <v>426</v>
       </c>
       <c r="C109" s="17" t="s">
-        <v>425</v>
+        <v>427</v>
       </c>
       <c r="D109" s="17" t="s">
-        <v>426</v>
+        <v>428</v>
       </c>
       <c r="E109" s="17" t="s">
-        <v>427</v>
+        <v>429</v>
       </c>
       <c r="F109" s="18"/>
       <c r="G109" s="18"/>
@@ -5381,19 +5395,19 @@
     </row>
     <row r="110" s="1" customFormat="1" ht="78.75" customHeight="1" spans="1:9">
       <c r="A110" s="16" t="s">
-        <v>428</v>
+        <v>430</v>
       </c>
       <c r="B110" s="16" t="s">
         <v>88</v>
       </c>
       <c r="C110" s="17" t="s">
-        <v>429</v>
+        <v>431</v>
       </c>
       <c r="D110" s="17" t="s">
-        <v>430</v>
+        <v>432</v>
       </c>
       <c r="E110" s="17" t="s">
-        <v>431</v>
+        <v>433</v>
       </c>
       <c r="F110" s="18"/>
       <c r="G110" s="18"/>
@@ -5402,19 +5416,19 @@
     </row>
     <row r="111" s="1" customFormat="1" ht="78.75" customHeight="1" spans="1:9">
       <c r="A111" s="16" t="s">
-        <v>432</v>
+        <v>434</v>
       </c>
       <c r="B111" s="16" t="s">
-        <v>433</v>
+        <v>435</v>
       </c>
       <c r="C111" s="17" t="s">
-        <v>434</v>
+        <v>436</v>
       </c>
       <c r="D111" s="17" t="s">
-        <v>435</v>
+        <v>437</v>
       </c>
       <c r="E111" s="17" t="s">
-        <v>436</v>
+        <v>438</v>
       </c>
       <c r="F111" s="18"/>
       <c r="G111" s="18"/>
@@ -5423,19 +5437,19 @@
     </row>
     <row r="112" s="1" customFormat="1" ht="78.75" customHeight="1" spans="1:9">
       <c r="A112" s="16" t="s">
-        <v>437</v>
+        <v>439</v>
       </c>
       <c r="B112" s="16" t="s">
-        <v>388</v>
+        <v>390</v>
       </c>
       <c r="C112" s="17" t="s">
-        <v>438</v>
+        <v>440</v>
       </c>
       <c r="D112" s="17" t="s">
-        <v>439</v>
+        <v>441</v>
       </c>
       <c r="E112" s="17" t="s">
-        <v>440</v>
+        <v>442</v>
       </c>
       <c r="F112" s="18"/>
       <c r="G112" s="18"/>
@@ -5444,26 +5458,26 @@
     </row>
     <row r="113" s="1" customFormat="1" ht="15.75" customHeight="1" spans="1:9">
       <c r="A113" s="14" t="s">
-        <v>441</v>
+        <v>443</v>
       </c>
       <c r="H113" s="15"/>
       <c r="I113" s="15"/>
     </row>
     <row r="114" s="1" customFormat="1" ht="78.75" customHeight="1" spans="1:9">
       <c r="A114" s="16" t="s">
-        <v>442</v>
+        <v>444</v>
       </c>
       <c r="B114" s="16" t="s">
-        <v>399</v>
+        <v>401</v>
       </c>
       <c r="C114" s="17" t="s">
-        <v>443</v>
+        <v>445</v>
       </c>
       <c r="D114" s="17" t="s">
-        <v>444</v>
+        <v>446</v>
       </c>
       <c r="E114" s="17" t="s">
-        <v>445</v>
+        <v>447</v>
       </c>
       <c r="F114" s="18"/>
       <c r="G114" s="18"/>
@@ -5472,26 +5486,26 @@
     </row>
     <row r="115" s="1" customFormat="1" ht="15.75" customHeight="1" spans="1:9">
       <c r="A115" s="14" t="s">
-        <v>446</v>
+        <v>448</v>
       </c>
       <c r="H115" s="15"/>
       <c r="I115" s="15"/>
     </row>
     <row r="116" s="1" customFormat="1" ht="173.25" customHeight="1" spans="1:9">
       <c r="A116" s="16" t="s">
-        <v>447</v>
+        <v>449</v>
       </c>
       <c r="B116" s="16" t="s">
-        <v>448</v>
+        <v>450</v>
       </c>
       <c r="C116" s="17" t="s">
-        <v>449</v>
+        <v>451</v>
       </c>
       <c r="D116" s="17" t="s">
-        <v>450</v>
+        <v>452</v>
       </c>
       <c r="E116" s="17" t="s">
-        <v>451</v>
+        <v>453</v>
       </c>
       <c r="F116" s="18"/>
       <c r="G116" s="18"/>
@@ -5500,19 +5514,19 @@
     </row>
     <row r="117" s="1" customFormat="1" ht="141.75" customHeight="1" spans="1:9">
       <c r="A117" s="16" t="s">
-        <v>452</v>
+        <v>454</v>
       </c>
       <c r="B117" s="16" t="s">
-        <v>453</v>
+        <v>455</v>
       </c>
       <c r="C117" s="17" t="s">
-        <v>454</v>
+        <v>456</v>
       </c>
       <c r="D117" s="17" t="s">
-        <v>455</v>
+        <v>457</v>
       </c>
       <c r="E117" s="17" t="s">
-        <v>456</v>
+        <v>458</v>
       </c>
       <c r="F117" s="18"/>
       <c r="G117" s="18"/>
@@ -5521,19 +5535,19 @@
     </row>
     <row r="118" s="1" customFormat="1" ht="157.5" customHeight="1" spans="1:9">
       <c r="A118" s="16" t="s">
-        <v>457</v>
+        <v>459</v>
       </c>
       <c r="B118" s="16" t="s">
-        <v>458</v>
+        <v>460</v>
       </c>
       <c r="C118" s="17" t="s">
-        <v>459</v>
+        <v>461</v>
       </c>
       <c r="D118" s="17" t="s">
-        <v>460</v>
+        <v>462</v>
       </c>
       <c r="E118" s="17" t="s">
-        <v>461</v>
+        <v>463</v>
       </c>
       <c r="F118" s="18"/>
       <c r="G118" s="18"/>
@@ -5542,19 +5556,19 @@
     </row>
     <row r="119" s="1" customFormat="1" ht="141.75" customHeight="1" spans="1:9">
       <c r="A119" s="16" t="s">
-        <v>462</v>
+        <v>464</v>
       </c>
       <c r="B119" s="16" t="s">
-        <v>463</v>
+        <v>465</v>
       </c>
       <c r="C119" s="17" t="s">
-        <v>464</v>
+        <v>466</v>
       </c>
       <c r="D119" s="17" t="s">
-        <v>465</v>
+        <v>467</v>
       </c>
       <c r="E119" s="17" t="s">
-        <v>466</v>
+        <v>468</v>
       </c>
       <c r="F119" s="18"/>
       <c r="G119" s="18"/>
@@ -5563,19 +5577,19 @@
     </row>
     <row r="120" s="1" customFormat="1" ht="141.75" customHeight="1" spans="1:9">
       <c r="A120" s="16" t="s">
-        <v>467</v>
+        <v>469</v>
       </c>
       <c r="B120" s="16" t="s">
         <v>128</v>
       </c>
       <c r="C120" s="17" t="s">
-        <v>468</v>
+        <v>470</v>
       </c>
       <c r="D120" s="17" t="s">
-        <v>469</v>
+        <v>471</v>
       </c>
       <c r="E120" s="17" t="s">
-        <v>470</v>
+        <v>472</v>
       </c>
       <c r="F120" s="18"/>
       <c r="G120" s="18"/>
@@ -5584,19 +5598,19 @@
     </row>
     <row r="121" s="1" customFormat="1" ht="78.75" customHeight="1" spans="1:9">
       <c r="A121" s="16" t="s">
-        <v>471</v>
+        <v>473</v>
       </c>
       <c r="B121" s="16" t="s">
-        <v>472</v>
+        <v>474</v>
       </c>
       <c r="C121" s="17" t="s">
-        <v>473</v>
+        <v>475</v>
       </c>
       <c r="D121" s="17" t="s">
-        <v>474</v>
+        <v>476</v>
       </c>
       <c r="E121" s="17" t="s">
-        <v>475</v>
+        <v>477</v>
       </c>
       <c r="F121" s="18"/>
       <c r="G121" s="18"/>
@@ -5605,26 +5619,26 @@
     </row>
     <row r="122" s="1" customFormat="1" ht="15.75" customHeight="1" spans="1:9">
       <c r="A122" s="14" t="s">
-        <v>476</v>
+        <v>478</v>
       </c>
       <c r="H122" s="15"/>
       <c r="I122" s="15"/>
     </row>
     <row r="123" s="1" customFormat="1" ht="78.75" customHeight="1" spans="1:9">
       <c r="A123" s="16" t="s">
-        <v>477</v>
+        <v>479</v>
       </c>
       <c r="B123" s="16" t="s">
-        <v>478</v>
+        <v>480</v>
       </c>
       <c r="C123" s="17" t="s">
-        <v>479</v>
+        <v>481</v>
       </c>
       <c r="D123" s="17" t="s">
-        <v>480</v>
+        <v>482</v>
       </c>
       <c r="E123" s="17" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
       <c r="F123" s="18"/>
       <c r="G123" s="18"/>
@@ -5633,19 +5647,19 @@
     </row>
     <row r="124" s="1" customFormat="1" ht="78.75" customHeight="1" spans="1:9">
       <c r="A124" s="16" t="s">
-        <v>482</v>
+        <v>484</v>
       </c>
       <c r="B124" s="16" t="s">
-        <v>472</v>
+        <v>474</v>
       </c>
       <c r="C124" s="17" t="s">
-        <v>483</v>
+        <v>485</v>
       </c>
       <c r="D124" s="17" t="s">
-        <v>484</v>
+        <v>486</v>
       </c>
       <c r="E124" s="17" t="s">
-        <v>485</v>
+        <v>487</v>
       </c>
       <c r="F124" s="18"/>
       <c r="G124" s="18"/>
@@ -5654,19 +5668,19 @@
     </row>
     <row r="125" s="1" customFormat="1" ht="78.75" customHeight="1" spans="1:9">
       <c r="A125" s="16" t="s">
-        <v>486</v>
+        <v>488</v>
       </c>
       <c r="B125" s="16" t="s">
-        <v>487</v>
+        <v>489</v>
       </c>
       <c r="C125" s="17" t="s">
-        <v>488</v>
+        <v>490</v>
       </c>
       <c r="D125" s="17" t="s">
-        <v>489</v>
+        <v>491</v>
       </c>
       <c r="E125" s="17" t="s">
-        <v>490</v>
+        <v>492</v>
       </c>
       <c r="F125" s="18"/>
       <c r="G125" s="18"/>
@@ -5675,19 +5689,19 @@
     </row>
     <row r="126" s="1" customFormat="1" ht="78.75" customHeight="1" spans="1:9">
       <c r="A126" s="16" t="s">
-        <v>491</v>
+        <v>493</v>
       </c>
       <c r="B126" s="16" t="s">
-        <v>383</v>
+        <v>385</v>
       </c>
       <c r="C126" s="17" t="s">
-        <v>492</v>
+        <v>494</v>
       </c>
       <c r="D126" s="17" t="s">
-        <v>493</v>
+        <v>495</v>
       </c>
       <c r="E126" s="17" t="s">
-        <v>494</v>
+        <v>496</v>
       </c>
       <c r="F126" s="18"/>
       <c r="G126" s="18"/>
@@ -5696,26 +5710,26 @@
     </row>
     <row r="127" s="1" customFormat="1" ht="15.75" customHeight="1" spans="1:9">
       <c r="A127" s="14" t="s">
-        <v>495</v>
+        <v>497</v>
       </c>
       <c r="H127" s="15"/>
       <c r="I127" s="15"/>
     </row>
     <row r="128" s="1" customFormat="1" ht="78.75" customHeight="1" spans="1:9">
       <c r="A128" s="16" t="s">
-        <v>496</v>
+        <v>498</v>
       </c>
       <c r="B128" s="16" t="s">
-        <v>497</v>
+        <v>499</v>
       </c>
       <c r="C128" s="17" t="s">
-        <v>498</v>
+        <v>500</v>
       </c>
       <c r="D128" s="17" t="s">
-        <v>499</v>
+        <v>501</v>
       </c>
       <c r="E128" s="17" t="s">
-        <v>500</v>
+        <v>502</v>
       </c>
       <c r="F128" s="18"/>
       <c r="G128" s="18"/>
@@ -5724,19 +5738,19 @@
     </row>
     <row r="129" s="1" customFormat="1" ht="78.75" customHeight="1" spans="1:9">
       <c r="A129" s="16" t="s">
-        <v>501</v>
+        <v>503</v>
       </c>
       <c r="B129" s="16" t="s">
-        <v>383</v>
+        <v>385</v>
       </c>
       <c r="C129" s="17" t="s">
-        <v>502</v>
+        <v>504</v>
       </c>
       <c r="D129" s="17" t="s">
-        <v>503</v>
+        <v>505</v>
       </c>
       <c r="E129" s="17" t="s">
-        <v>504</v>
+        <v>506</v>
       </c>
       <c r="F129" s="18"/>
       <c r="G129" s="18"/>
@@ -5745,19 +5759,19 @@
     </row>
     <row r="130" s="1" customFormat="1" ht="78.75" customHeight="1" spans="1:9">
       <c r="A130" s="16" t="s">
-        <v>505</v>
+        <v>507</v>
       </c>
       <c r="B130" s="16" t="s">
-        <v>506</v>
+        <v>508</v>
       </c>
       <c r="C130" s="17" t="s">
-        <v>507</v>
+        <v>509</v>
       </c>
       <c r="D130" s="17" t="s">
-        <v>508</v>
+        <v>510</v>
       </c>
       <c r="E130" s="17" t="s">
-        <v>509</v>
+        <v>511</v>
       </c>
       <c r="F130" s="18"/>
       <c r="G130" s="18"/>
@@ -5766,26 +5780,26 @@
     </row>
     <row r="131" s="1" customFormat="1" ht="15.75" customHeight="1" spans="1:9">
       <c r="A131" s="14" t="s">
-        <v>510</v>
+        <v>512</v>
       </c>
       <c r="H131" s="15"/>
       <c r="I131" s="15"/>
     </row>
     <row r="132" s="1" customFormat="1" ht="157.5" customHeight="1" spans="1:9">
       <c r="A132" s="17" t="s">
-        <v>511</v>
+        <v>513</v>
       </c>
       <c r="B132" s="17" t="s">
-        <v>512</v>
+        <v>514</v>
       </c>
       <c r="C132" s="17" t="s">
-        <v>513</v>
+        <v>515</v>
       </c>
       <c r="D132" s="17" t="s">
-        <v>514</v>
+        <v>516</v>
       </c>
       <c r="E132" s="17" t="s">
-        <v>515</v>
+        <v>517</v>
       </c>
       <c r="F132" s="18"/>
       <c r="G132" s="18"/>
@@ -5794,19 +5808,19 @@
     </row>
     <row r="133" s="1" customFormat="1" ht="220.5" customHeight="1" spans="1:9">
       <c r="A133" s="16" t="s">
-        <v>516</v>
+        <v>518</v>
       </c>
       <c r="B133" s="16" t="s">
-        <v>517</v>
+        <v>519</v>
       </c>
       <c r="C133" s="17" t="s">
-        <v>518</v>
+        <v>520</v>
       </c>
       <c r="D133" s="17" t="s">
-        <v>519</v>
+        <v>521</v>
       </c>
       <c r="E133" s="17" t="s">
-        <v>520</v>
+        <v>522</v>
       </c>
       <c r="F133" s="18"/>
       <c r="G133" s="18"/>
@@ -5815,19 +5829,19 @@
     </row>
     <row r="134" s="1" customFormat="1" ht="94.5" customHeight="1" spans="1:9">
       <c r="A134" s="17" t="s">
-        <v>521</v>
+        <v>523</v>
       </c>
       <c r="B134" s="17" t="s">
-        <v>522</v>
+        <v>524</v>
       </c>
       <c r="C134" s="17" t="s">
-        <v>523</v>
+        <v>525</v>
       </c>
       <c r="D134" s="17" t="s">
-        <v>524</v>
+        <v>526</v>
       </c>
       <c r="E134" s="17" t="s">
-        <v>525</v>
+        <v>527</v>
       </c>
       <c r="F134" s="18"/>
       <c r="G134" s="18"/>
@@ -5836,19 +5850,19 @@
     </row>
     <row r="135" s="1" customFormat="1" ht="141.75" customHeight="1" spans="1:9">
       <c r="A135" s="17" t="s">
-        <v>526</v>
+        <v>528</v>
       </c>
       <c r="B135" s="17" t="s">
-        <v>522</v>
+        <v>524</v>
       </c>
       <c r="C135" s="17" t="s">
-        <v>527</v>
+        <v>529</v>
       </c>
       <c r="D135" s="17" t="s">
-        <v>528</v>
+        <v>530</v>
       </c>
       <c r="E135" s="17" t="s">
-        <v>529</v>
+        <v>531</v>
       </c>
       <c r="F135" s="18"/>
       <c r="G135" s="18"/>
@@ -5857,19 +5871,19 @@
     </row>
     <row r="136" s="1" customFormat="1" ht="78.75" customHeight="1" spans="1:9">
       <c r="A136" s="16" t="s">
-        <v>530</v>
+        <v>532</v>
       </c>
       <c r="B136" s="16" t="s">
-        <v>531</v>
+        <v>533</v>
       </c>
       <c r="C136" s="17" t="s">
-        <v>532</v>
+        <v>534</v>
       </c>
       <c r="D136" s="17" t="s">
-        <v>533</v>
+        <v>535</v>
       </c>
       <c r="E136" s="17" t="s">
-        <v>534</v>
+        <v>536</v>
       </c>
       <c r="F136" s="18"/>
       <c r="G136" s="18"/>
@@ -5878,26 +5892,26 @@
     </row>
     <row r="137" s="1" customFormat="1" ht="15.75" customHeight="1" spans="1:9">
       <c r="A137" s="14" t="s">
-        <v>535</v>
+        <v>537</v>
       </c>
       <c r="H137" s="15"/>
       <c r="I137" s="15"/>
     </row>
     <row r="138" s="1" customFormat="1" ht="94.5" customHeight="1" spans="1:9">
       <c r="A138" s="16" t="s">
-        <v>536</v>
+        <v>538</v>
       </c>
       <c r="B138" s="16" t="s">
-        <v>537</v>
+        <v>539</v>
       </c>
       <c r="C138" s="17" t="s">
-        <v>538</v>
-      </c>
-      <c r="D138" s="20" t="s">
-        <v>539</v>
+        <v>540</v>
+      </c>
+      <c r="D138" s="21" t="s">
+        <v>541</v>
       </c>
       <c r="E138" s="17" t="s">
-        <v>540</v>
+        <v>542</v>
       </c>
       <c r="F138" s="18"/>
       <c r="G138" s="18"/>
@@ -5906,19 +5920,19 @@
     </row>
     <row r="139" s="1" customFormat="1" ht="94.5" customHeight="1" spans="1:9">
       <c r="A139" s="16" t="s">
-        <v>541</v>
+        <v>543</v>
       </c>
       <c r="B139" s="16" t="s">
-        <v>542</v>
+        <v>544</v>
       </c>
       <c r="C139" s="17" t="s">
-        <v>543</v>
+        <v>545</v>
       </c>
       <c r="D139" s="20" t="s">
-        <v>544</v>
+        <v>546</v>
       </c>
       <c r="E139" s="17" t="s">
-        <v>545</v>
+        <v>547</v>
       </c>
       <c r="F139" s="18"/>
       <c r="G139" s="18"/>
@@ -5927,19 +5941,19 @@
     </row>
     <row r="140" s="1" customFormat="1" ht="157.5" customHeight="1" spans="1:9">
       <c r="A140" s="16" t="s">
-        <v>546</v>
+        <v>548</v>
       </c>
       <c r="B140" s="16" t="s">
-        <v>537</v>
+        <v>539</v>
       </c>
       <c r="C140" s="17" t="s">
-        <v>547</v>
+        <v>549</v>
       </c>
       <c r="D140" s="20" t="s">
-        <v>548</v>
+        <v>550</v>
       </c>
       <c r="E140" s="17" t="s">
-        <v>549</v>
+        <v>551</v>
       </c>
       <c r="F140" s="18"/>
       <c r="G140" s="18"/>
@@ -5948,19 +5962,19 @@
     </row>
     <row r="141" s="1" customFormat="1" ht="220.5" customHeight="1" spans="1:9">
       <c r="A141" s="16" t="s">
-        <v>550</v>
+        <v>552</v>
       </c>
       <c r="B141" s="16" t="s">
-        <v>537</v>
+        <v>539</v>
       </c>
       <c r="C141" s="17" t="s">
-        <v>551</v>
+        <v>553</v>
       </c>
       <c r="D141" s="17" t="s">
-        <v>552</v>
+        <v>554</v>
       </c>
       <c r="E141" s="17" t="s">
-        <v>553</v>
+        <v>555</v>
       </c>
       <c r="F141" s="18"/>
       <c r="G141" s="18"/>
@@ -5969,19 +5983,19 @@
     </row>
     <row r="142" s="1" customFormat="1" ht="141.75" customHeight="1" spans="1:9">
       <c r="A142" s="16" t="s">
-        <v>554</v>
+        <v>556</v>
       </c>
       <c r="B142" s="16" t="s">
-        <v>537</v>
+        <v>539</v>
       </c>
       <c r="C142" s="17" t="s">
-        <v>555</v>
+        <v>557</v>
       </c>
       <c r="D142" s="20" t="s">
-        <v>556</v>
+        <v>558</v>
       </c>
       <c r="E142" s="17" t="s">
-        <v>557</v>
+        <v>559</v>
       </c>
       <c r="F142" s="18"/>
       <c r="G142" s="18"/>
@@ -5990,19 +6004,19 @@
     </row>
     <row r="143" s="1" customFormat="1" ht="141.75" customHeight="1" spans="1:9">
       <c r="A143" s="16" t="s">
-        <v>558</v>
+        <v>560</v>
       </c>
       <c r="B143" s="16" t="s">
-        <v>537</v>
+        <v>539</v>
       </c>
       <c r="C143" s="17" t="s">
-        <v>559</v>
+        <v>561</v>
       </c>
       <c r="D143" s="20" t="s">
-        <v>560</v>
+        <v>562</v>
       </c>
       <c r="E143" s="17" t="s">
-        <v>561</v>
+        <v>563</v>
       </c>
       <c r="F143" s="18"/>
       <c r="G143" s="18"/>
@@ -6011,19 +6025,19 @@
     </row>
     <row r="144" s="1" customFormat="1" ht="204.75" customHeight="1" spans="1:9">
       <c r="A144" s="16" t="s">
-        <v>562</v>
+        <v>564</v>
       </c>
       <c r="B144" s="16" t="s">
-        <v>537</v>
+        <v>539</v>
       </c>
       <c r="C144" s="17" t="s">
-        <v>563</v>
+        <v>565</v>
       </c>
       <c r="D144" s="20" t="s">
-        <v>564</v>
+        <v>566</v>
       </c>
       <c r="E144" s="17" t="s">
-        <v>565</v>
+        <v>567</v>
       </c>
       <c r="F144" s="18"/>
       <c r="G144" s="18"/>
@@ -6032,26 +6046,26 @@
     </row>
     <row r="145" s="1" customFormat="1" ht="15.75" customHeight="1" spans="1:9">
       <c r="A145" s="14" t="s">
-        <v>566</v>
+        <v>568</v>
       </c>
       <c r="H145" s="15"/>
       <c r="I145" s="15"/>
     </row>
     <row r="146" s="1" customFormat="1" ht="78.75" customHeight="1" spans="1:9">
       <c r="A146" s="16" t="s">
-        <v>567</v>
+        <v>569</v>
       </c>
       <c r="B146" s="16" t="s">
-        <v>568</v>
+        <v>570</v>
       </c>
       <c r="C146" s="17" t="s">
-        <v>569</v>
+        <v>571</v>
       </c>
       <c r="D146" s="17" t="s">
-        <v>570</v>
+        <v>572</v>
       </c>
       <c r="E146" s="17" t="s">
-        <v>571</v>
+        <v>573</v>
       </c>
       <c r="F146" s="18"/>
       <c r="G146" s="18"/>
@@ -6060,19 +6074,19 @@
     </row>
     <row r="147" s="1" customFormat="1" ht="78.75" customHeight="1" spans="1:9">
       <c r="A147" s="16" t="s">
-        <v>572</v>
+        <v>574</v>
       </c>
       <c r="B147" s="16" t="s">
-        <v>573</v>
+        <v>575</v>
       </c>
       <c r="C147" s="17" t="s">
-        <v>574</v>
+        <v>576</v>
       </c>
       <c r="D147" s="17" t="s">
-        <v>575</v>
+        <v>577</v>
       </c>
       <c r="E147" s="17" t="s">
-        <v>576</v>
+        <v>578</v>
       </c>
       <c r="F147" s="18"/>
       <c r="G147" s="18"/>
@@ -6081,26 +6095,26 @@
     </row>
     <row r="148" s="1" customFormat="1" ht="15.75" customHeight="1" spans="1:9">
       <c r="A148" s="14" t="s">
-        <v>577</v>
+        <v>579</v>
       </c>
       <c r="H148" s="15"/>
       <c r="I148" s="15"/>
     </row>
     <row r="149" s="1" customFormat="1" ht="126" customHeight="1" spans="1:9">
       <c r="A149" s="16" t="s">
-        <v>578</v>
+        <v>580</v>
       </c>
       <c r="B149" s="16" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="C149" s="17" t="s">
-        <v>579</v>
+        <v>581</v>
       </c>
       <c r="D149" s="17" t="s">
-        <v>580</v>
+        <v>582</v>
       </c>
       <c r="E149" s="17" t="s">
-        <v>581</v>
+        <v>583</v>
       </c>
       <c r="F149" s="18"/>
       <c r="G149" s="18"/>
@@ -6109,19 +6123,19 @@
     </row>
     <row r="150" s="1" customFormat="1" ht="157.5" customHeight="1" spans="1:9">
       <c r="A150" s="16" t="s">
-        <v>582</v>
+        <v>584</v>
       </c>
       <c r="B150" s="16" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="C150" s="17" t="s">
-        <v>583</v>
+        <v>585</v>
       </c>
       <c r="D150" s="17" t="s">
-        <v>584</v>
+        <v>586</v>
       </c>
       <c r="E150" s="17" t="s">
-        <v>585</v>
+        <v>587</v>
       </c>
       <c r="F150" s="18"/>
       <c r="G150" s="18"/>
@@ -6130,19 +6144,19 @@
     </row>
     <row r="151" s="1" customFormat="1" ht="189" customHeight="1" spans="1:9">
       <c r="A151" s="16" t="s">
-        <v>586</v>
+        <v>588</v>
       </c>
       <c r="B151" s="16" t="s">
-        <v>587</v>
+        <v>589</v>
       </c>
       <c r="C151" s="17" t="s">
-        <v>588</v>
+        <v>590</v>
       </c>
       <c r="D151" s="17" t="s">
-        <v>589</v>
+        <v>591</v>
       </c>
       <c r="E151" s="17" t="s">
-        <v>590</v>
+        <v>592</v>
       </c>
       <c r="F151" s="18"/>
       <c r="G151" s="18"/>
@@ -6151,19 +6165,19 @@
     </row>
     <row r="152" s="1" customFormat="1" ht="157.5" customHeight="1" spans="1:9">
       <c r="A152" s="16" t="s">
-        <v>591</v>
+        <v>593</v>
       </c>
       <c r="B152" s="16" t="s">
-        <v>587</v>
+        <v>589</v>
       </c>
       <c r="C152" s="17" t="s">
-        <v>592</v>
+        <v>594</v>
       </c>
       <c r="D152" s="17" t="s">
-        <v>593</v>
+        <v>595</v>
       </c>
       <c r="E152" s="17" t="s">
-        <v>594</v>
+        <v>596</v>
       </c>
       <c r="F152" s="18"/>
       <c r="G152" s="18"/>
@@ -6172,19 +6186,19 @@
     </row>
     <row r="153" s="1" customFormat="1" ht="141.75" customHeight="1" spans="1:9">
       <c r="A153" s="16" t="s">
-        <v>595</v>
+        <v>597</v>
       </c>
       <c r="B153" s="16" t="s">
-        <v>596</v>
+        <v>598</v>
       </c>
       <c r="C153" s="17" t="s">
-        <v>597</v>
+        <v>599</v>
       </c>
       <c r="D153" s="17" t="s">
-        <v>598</v>
+        <v>600</v>
       </c>
       <c r="E153" s="17" t="s">
-        <v>599</v>
+        <v>601</v>
       </c>
       <c r="F153" s="18"/>
       <c r="G153" s="18"/>
@@ -6193,19 +6207,19 @@
     </row>
     <row r="154" ht="189" customHeight="1" spans="1:9">
       <c r="A154" s="16" t="s">
-        <v>600</v>
+        <v>602</v>
       </c>
       <c r="B154" s="16" t="s">
-        <v>601</v>
+        <v>603</v>
       </c>
       <c r="C154" s="17" t="s">
-        <v>602</v>
+        <v>604</v>
       </c>
       <c r="D154" s="17" t="s">
-        <v>603</v>
+        <v>605</v>
       </c>
       <c r="E154" s="17" t="s">
-        <v>604</v>
+        <v>606</v>
       </c>
       <c r="F154" s="18"/>
       <c r="G154" s="18"/>
@@ -6214,17 +6228,17 @@
     </row>
     <row r="155" ht="15.75" customHeight="1" spans="1:9">
       <c r="A155" s="14" t="s">
-        <v>605</v>
+        <v>607</v>
       </c>
       <c r="H155" s="15"/>
       <c r="I155" s="15"/>
     </row>
     <row r="156" ht="157.5" customHeight="1" spans="1:9">
       <c r="A156" s="16" t="s">
-        <v>606</v>
+        <v>608</v>
       </c>
       <c r="B156" s="16" t="s">
-        <v>537</v>
+        <v>539</v>
       </c>
       <c r="C156" s="17" t="s">
         <v>254</v>
@@ -6233,7 +6247,7 @@
         <v>255</v>
       </c>
       <c r="E156" s="17" t="s">
-        <v>607</v>
+        <v>609</v>
       </c>
       <c r="F156" s="18"/>
       <c r="G156" s="18"/>
@@ -6242,19 +6256,19 @@
     </row>
     <row r="157" ht="252" customHeight="1" spans="1:9">
       <c r="A157" s="16" t="s">
-        <v>608</v>
+        <v>610</v>
       </c>
       <c r="B157" s="16" t="s">
-        <v>609</v>
+        <v>611</v>
       </c>
       <c r="C157" s="17" t="s">
-        <v>610</v>
+        <v>612</v>
       </c>
       <c r="D157" s="17" t="s">
-        <v>611</v>
+        <v>613</v>
       </c>
       <c r="E157" s="17" t="s">
-        <v>612</v>
+        <v>614</v>
       </c>
       <c r="F157" s="18"/>
       <c r="G157" s="18"/>
@@ -6263,19 +6277,19 @@
     </row>
     <row r="158" ht="220.5" customHeight="1" spans="1:9">
       <c r="A158" s="16" t="s">
-        <v>613</v>
+        <v>615</v>
       </c>
       <c r="B158" s="16" t="s">
-        <v>609</v>
+        <v>611</v>
       </c>
       <c r="C158" s="17" t="s">
-        <v>614</v>
+        <v>616</v>
       </c>
       <c r="D158" s="17" t="s">
-        <v>615</v>
+        <v>617</v>
       </c>
       <c r="E158" s="17" t="s">
-        <v>616</v>
+        <v>618</v>
       </c>
       <c r="F158" s="18"/>
       <c r="G158" s="18"/>
@@ -6284,19 +6298,19 @@
     </row>
     <row r="159" ht="204.75" customHeight="1" spans="1:9">
       <c r="A159" s="17" t="s">
-        <v>617</v>
+        <v>619</v>
       </c>
       <c r="B159" s="17" t="s">
         <v>104</v>
       </c>
       <c r="C159" s="17" t="s">
-        <v>618</v>
+        <v>620</v>
       </c>
       <c r="D159" s="17" t="s">
         <v>238</v>
       </c>
       <c r="E159" s="17" t="s">
-        <v>619</v>
+        <v>621</v>
       </c>
       <c r="F159" s="18"/>
       <c r="G159" s="18"/>
@@ -6305,19 +6319,19 @@
     </row>
     <row r="160" ht="126" customHeight="1" spans="1:9">
       <c r="A160" s="16" t="s">
-        <v>620</v>
+        <v>622</v>
       </c>
       <c r="B160" s="16" t="s">
-        <v>537</v>
+        <v>539</v>
       </c>
       <c r="C160" s="17" t="s">
-        <v>621</v>
+        <v>623</v>
       </c>
       <c r="D160" s="17" t="s">
-        <v>622</v>
+        <v>624</v>
       </c>
       <c r="E160" s="17" t="s">
-        <v>623</v>
+        <v>625</v>
       </c>
       <c r="F160" s="18"/>
       <c r="G160" s="18"/>
@@ -6326,19 +6340,19 @@
     </row>
     <row r="161" ht="78.75" customHeight="1" spans="1:9">
       <c r="A161" s="16" t="s">
-        <v>624</v>
+        <v>626</v>
       </c>
       <c r="B161" s="16" t="s">
-        <v>399</v>
+        <v>401</v>
       </c>
       <c r="C161" s="17" t="s">
-        <v>625</v>
+        <v>627</v>
       </c>
       <c r="D161" s="17" t="s">
-        <v>626</v>
+        <v>628</v>
       </c>
       <c r="E161" s="17" t="s">
-        <v>627</v>
+        <v>629</v>
       </c>
       <c r="F161" s="18"/>
       <c r="G161" s="18"/>
@@ -6347,26 +6361,26 @@
     </row>
     <row r="162" ht="15.75" customHeight="1" spans="1:9">
       <c r="A162" s="14" t="s">
-        <v>628</v>
+        <v>630</v>
       </c>
       <c r="H162" s="15"/>
       <c r="I162" s="15"/>
     </row>
     <row r="163" ht="157.5" customHeight="1" spans="1:9">
       <c r="A163" s="16" t="s">
-        <v>629</v>
+        <v>631</v>
       </c>
       <c r="B163" s="16" t="s">
-        <v>630</v>
+        <v>632</v>
       </c>
       <c r="C163" s="17" t="s">
-        <v>631</v>
+        <v>633</v>
       </c>
       <c r="D163" s="17" t="s">
-        <v>632</v>
+        <v>634</v>
       </c>
       <c r="E163" s="17" t="s">
-        <v>633</v>
+        <v>635</v>
       </c>
       <c r="F163" s="18"/>
       <c r="G163" s="18"/>

</xml_diff>